<commit_message>
Added no decimal validation to toal booked units in supplier sheet
</commit_message>
<xml_diff>
--- a/samples/Supplier PO sheet-DDMMYYYY.xlsx
+++ b/samples/Supplier PO sheet-DDMMYYYY.xlsx
@@ -1977,6 +1977,7 @@
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
+      <c r="E3" s="15"/>
       <c r="F3" s="15">
         <v>1</v>
       </c>
@@ -2019,6 +2020,7 @@
       </c>
       <c r="C4" s="25"/>
       <c r="D4" s="25"/>
+      <c r="E4" s="15"/>
       <c r="F4" s="15">
         <v>1</v>
       </c>
@@ -2061,6 +2063,7 @@
       </c>
       <c r="C5" s="25"/>
       <c r="D5" s="25"/>
+      <c r="E5" s="15"/>
       <c r="F5" s="15">
         <v>1</v>
       </c>
@@ -2103,6 +2106,7 @@
       </c>
       <c r="C6" s="25"/>
       <c r="D6" s="25"/>
+      <c r="E6" s="15"/>
       <c r="F6" s="15">
         <v>1</v>
       </c>
@@ -2145,6 +2149,7 @@
       </c>
       <c r="C7" s="25"/>
       <c r="D7" s="25"/>
+      <c r="E7" s="15"/>
       <c r="F7" s="15">
         <v>1</v>
       </c>
@@ -2187,6 +2192,7 @@
       </c>
       <c r="C8" s="25"/>
       <c r="D8" s="25"/>
+      <c r="E8" s="15"/>
       <c r="F8" s="15">
         <v>1</v>
       </c>
@@ -2229,6 +2235,7 @@
       </c>
       <c r="C9" s="25"/>
       <c r="D9" s="25"/>
+      <c r="E9" s="15"/>
       <c r="F9" s="15">
         <v>1</v>
       </c>
@@ -2271,6 +2278,7 @@
       </c>
       <c r="C10" s="25"/>
       <c r="D10" s="25"/>
+      <c r="E10" s="15"/>
       <c r="F10" s="15">
         <v>1</v>
       </c>
@@ -2313,6 +2321,7 @@
       </c>
       <c r="C11" s="25"/>
       <c r="D11" s="25"/>
+      <c r="E11" s="15"/>
       <c r="F11" s="15">
         <v>1</v>
       </c>
@@ -2355,6 +2364,7 @@
       </c>
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
+      <c r="E12" s="15"/>
       <c r="F12" s="15">
         <v>1</v>
       </c>
@@ -2397,6 +2407,7 @@
       </c>
       <c r="C13" s="25"/>
       <c r="D13" s="25"/>
+      <c r="E13" s="15"/>
       <c r="F13" s="15">
         <v>1</v>
       </c>
@@ -2439,6 +2450,7 @@
       </c>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
+      <c r="E14" s="15"/>
       <c r="F14" s="15">
         <v>1</v>
       </c>
@@ -2481,6 +2493,7 @@
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
+      <c r="E15" s="15"/>
       <c r="F15" s="15">
         <v>1</v>
       </c>
@@ -2523,6 +2536,7 @@
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
+      <c r="E16" s="15"/>
       <c r="F16" s="15">
         <v>1</v>
       </c>
@@ -2565,6 +2579,7 @@
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="25"/>
+      <c r="E17" s="15"/>
       <c r="F17" s="15">
         <v>1</v>
       </c>
@@ -2607,6 +2622,7 @@
       </c>
       <c r="C18" s="25"/>
       <c r="D18" s="25"/>
+      <c r="E18" s="15"/>
       <c r="F18" s="15">
         <v>1</v>
       </c>
@@ -2649,6 +2665,7 @@
       </c>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
+      <c r="E19" s="15"/>
       <c r="F19" s="15">
         <v>1</v>
       </c>
@@ -2691,6 +2708,7 @@
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
+      <c r="E20" s="15"/>
       <c r="F20" s="15">
         <v>1</v>
       </c>
@@ -2733,6 +2751,7 @@
       </c>
       <c r="C21" s="25"/>
       <c r="D21" s="25"/>
+      <c r="E21" s="15"/>
       <c r="F21" s="15">
         <v>1</v>
       </c>
@@ -2775,6 +2794,7 @@
       </c>
       <c r="C22" s="25"/>
       <c r="D22" s="25"/>
+      <c r="E22" s="15"/>
       <c r="F22" s="15">
         <v>1</v>
       </c>
@@ -2817,6 +2837,7 @@
       </c>
       <c r="C23" s="25"/>
       <c r="D23" s="25"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="15">
         <v>1</v>
       </c>
@@ -2859,6 +2880,7 @@
       </c>
       <c r="C24" s="25"/>
       <c r="D24" s="25"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="15">
         <v>1</v>
       </c>
@@ -2901,6 +2923,7 @@
       </c>
       <c r="C25" s="25"/>
       <c r="D25" s="25"/>
+      <c r="E25" s="15"/>
       <c r="F25" s="15">
         <v>1</v>
       </c>
@@ -2943,6 +2966,7 @@
       </c>
       <c r="C26" s="25"/>
       <c r="D26" s="25"/>
+      <c r="E26" s="15"/>
       <c r="F26" s="15">
         <v>1</v>
       </c>
@@ -2985,6 +3009,7 @@
       </c>
       <c r="C27" s="25"/>
       <c r="D27" s="25"/>
+      <c r="E27" s="15"/>
       <c r="F27" s="15">
         <v>1</v>
       </c>
@@ -3027,6 +3052,7 @@
       </c>
       <c r="C28" s="25"/>
       <c r="D28" s="25"/>
+      <c r="E28" s="15"/>
       <c r="F28" s="15">
         <v>1</v>
       </c>
@@ -3069,6 +3095,7 @@
       </c>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
+      <c r="E29" s="15"/>
       <c r="F29" s="15">
         <v>1</v>
       </c>
@@ -3111,6 +3138,7 @@
       </c>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
+      <c r="E30" s="15"/>
       <c r="F30" s="15">
         <v>1</v>
       </c>
@@ -3153,6 +3181,7 @@
       </c>
       <c r="C31" s="25"/>
       <c r="D31" s="25"/>
+      <c r="E31" s="15"/>
       <c r="F31" s="15">
         <v>1</v>
       </c>
@@ -3195,6 +3224,7 @@
       </c>
       <c r="C32" s="25"/>
       <c r="D32" s="25"/>
+      <c r="E32" s="15"/>
       <c r="F32" s="15">
         <v>1</v>
       </c>
@@ -3237,6 +3267,7 @@
       </c>
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
+      <c r="E33" s="15"/>
       <c r="F33" s="15">
         <v>1</v>
       </c>
@@ -3279,6 +3310,7 @@
       </c>
       <c r="C34" s="25"/>
       <c r="D34" s="25"/>
+      <c r="E34" s="15"/>
       <c r="F34" s="15">
         <v>1</v>
       </c>
@@ -3321,6 +3353,7 @@
       </c>
       <c r="C35" s="25"/>
       <c r="D35" s="25"/>
+      <c r="E35" s="15"/>
       <c r="F35" s="15">
         <v>1</v>
       </c>
@@ -3363,6 +3396,7 @@
       </c>
       <c r="C36" s="25"/>
       <c r="D36" s="25"/>
+      <c r="E36" s="15"/>
       <c r="F36" s="15">
         <v>1</v>
       </c>
@@ -3405,6 +3439,7 @@
       </c>
       <c r="C37" s="25"/>
       <c r="D37" s="25"/>
+      <c r="E37" s="15"/>
       <c r="F37" s="15">
         <v>1</v>
       </c>
@@ -3447,6 +3482,7 @@
       </c>
       <c r="C38" s="25"/>
       <c r="D38" s="25"/>
+      <c r="E38" s="15"/>
       <c r="F38" s="15">
         <v>1</v>
       </c>
@@ -3489,6 +3525,7 @@
       </c>
       <c r="C39" s="25"/>
       <c r="D39" s="25"/>
+      <c r="E39" s="15"/>
       <c r="F39" s="15">
         <v>1</v>
       </c>
@@ -3531,6 +3568,7 @@
       </c>
       <c r="C40" s="25"/>
       <c r="D40" s="25"/>
+      <c r="E40" s="15"/>
       <c r="F40" s="15">
         <v>1</v>
       </c>
@@ -3573,6 +3611,7 @@
       </c>
       <c r="C41" s="25"/>
       <c r="D41" s="25"/>
+      <c r="E41" s="15"/>
       <c r="F41" s="15">
         <v>1</v>
       </c>
@@ -3615,6 +3654,7 @@
       </c>
       <c r="C42" s="25"/>
       <c r="D42" s="25"/>
+      <c r="E42" s="15"/>
       <c r="F42" s="15">
         <v>1</v>
       </c>
@@ -3657,6 +3697,7 @@
       </c>
       <c r="C43" s="25"/>
       <c r="D43" s="25"/>
+      <c r="E43" s="15"/>
       <c r="F43" s="15">
         <v>1</v>
       </c>
@@ -3699,6 +3740,7 @@
       </c>
       <c r="C44" s="25"/>
       <c r="D44" s="25"/>
+      <c r="E44" s="15"/>
       <c r="F44" s="15">
         <v>1</v>
       </c>
@@ -3741,6 +3783,7 @@
       </c>
       <c r="C45" s="25"/>
       <c r="D45" s="25"/>
+      <c r="E45" s="15"/>
       <c r="F45" s="15">
         <v>1</v>
       </c>
@@ -3783,6 +3826,7 @@
       </c>
       <c r="C46" s="25"/>
       <c r="D46" s="25"/>
+      <c r="E46" s="15"/>
       <c r="F46" s="15">
         <v>1</v>
       </c>
@@ -3825,6 +3869,7 @@
       </c>
       <c r="C47" s="25"/>
       <c r="D47" s="25"/>
+      <c r="E47" s="15"/>
       <c r="F47" s="15">
         <v>1</v>
       </c>
@@ -3867,6 +3912,7 @@
       </c>
       <c r="C48" s="25"/>
       <c r="D48" s="25"/>
+      <c r="E48" s="15"/>
       <c r="F48" s="15">
         <v>1</v>
       </c>
@@ -3909,6 +3955,7 @@
       </c>
       <c r="C49" s="25"/>
       <c r="D49" s="25"/>
+      <c r="E49" s="15"/>
       <c r="F49" s="15">
         <v>1</v>
       </c>
@@ -3951,6 +3998,7 @@
       </c>
       <c r="C50" s="25"/>
       <c r="D50" s="25"/>
+      <c r="E50" s="15"/>
       <c r="F50" s="15">
         <v>1</v>
       </c>
@@ -3993,6 +4041,7 @@
       </c>
       <c r="C51" s="25"/>
       <c r="D51" s="25"/>
+      <c r="E51" s="15"/>
       <c r="F51" s="15">
         <v>1</v>
       </c>
@@ -4035,6 +4084,7 @@
       </c>
       <c r="C52" s="25"/>
       <c r="D52" s="25"/>
+      <c r="E52" s="15"/>
       <c r="F52" s="15">
         <v>1</v>
       </c>
@@ -4077,6 +4127,7 @@
       </c>
       <c r="C53" s="25"/>
       <c r="D53" s="25"/>
+      <c r="E53" s="15"/>
       <c r="F53" s="15">
         <v>1</v>
       </c>
@@ -4119,6 +4170,7 @@
       </c>
       <c r="C54" s="25"/>
       <c r="D54" s="25"/>
+      <c r="E54" s="15"/>
       <c r="F54" s="15">
         <v>1</v>
       </c>
@@ -4161,6 +4213,7 @@
       </c>
       <c r="C55" s="25"/>
       <c r="D55" s="25"/>
+      <c r="E55" s="15"/>
       <c r="F55" s="15">
         <v>1</v>
       </c>
@@ -4203,6 +4256,7 @@
       </c>
       <c r="C56" s="25"/>
       <c r="D56" s="25"/>
+      <c r="E56" s="15"/>
       <c r="F56" s="15">
         <v>1</v>
       </c>
@@ -4245,6 +4299,7 @@
       </c>
       <c r="C57" s="25"/>
       <c r="D57" s="25"/>
+      <c r="E57" s="15"/>
       <c r="F57" s="15">
         <v>1</v>
       </c>
@@ -4287,6 +4342,7 @@
       </c>
       <c r="C58" s="25"/>
       <c r="D58" s="25"/>
+      <c r="E58" s="15"/>
       <c r="F58" s="15">
         <v>1</v>
       </c>
@@ -4329,6 +4385,7 @@
       </c>
       <c r="C59" s="25"/>
       <c r="D59" s="25"/>
+      <c r="E59" s="15"/>
       <c r="F59" s="15">
         <v>1</v>
       </c>
@@ -4371,6 +4428,7 @@
       </c>
       <c r="C60" s="25"/>
       <c r="D60" s="25"/>
+      <c r="E60" s="15"/>
       <c r="F60" s="15">
         <v>1</v>
       </c>
@@ -4413,6 +4471,7 @@
       </c>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
+      <c r="E61" s="15"/>
       <c r="F61" s="15">
         <v>1</v>
       </c>
@@ -4455,6 +4514,7 @@
       </c>
       <c r="C62" s="25"/>
       <c r="D62" s="25"/>
+      <c r="E62" s="15"/>
       <c r="F62" s="15">
         <v>1</v>
       </c>
@@ -4497,6 +4557,7 @@
       </c>
       <c r="C63" s="25"/>
       <c r="D63" s="25"/>
+      <c r="E63" s="15"/>
       <c r="F63" s="15">
         <v>1</v>
       </c>
@@ -4539,6 +4600,7 @@
       </c>
       <c r="C64" s="25"/>
       <c r="D64" s="25"/>
+      <c r="E64" s="15"/>
       <c r="F64" s="15">
         <v>1</v>
       </c>
@@ -4581,6 +4643,7 @@
       </c>
       <c r="C65" s="25"/>
       <c r="D65" s="25"/>
+      <c r="E65" s="15"/>
       <c r="F65" s="15">
         <v>1</v>
       </c>
@@ -4623,6 +4686,7 @@
       </c>
       <c r="C66" s="25"/>
       <c r="D66" s="25"/>
+      <c r="E66" s="15"/>
       <c r="F66" s="15">
         <v>1</v>
       </c>
@@ -4665,6 +4729,7 @@
       </c>
       <c r="C67" s="25"/>
       <c r="D67" s="25"/>
+      <c r="E67" s="15"/>
       <c r="F67" s="15">
         <v>1</v>
       </c>
@@ -4707,6 +4772,7 @@
       </c>
       <c r="C68" s="25"/>
       <c r="D68" s="25"/>
+      <c r="E68" s="15"/>
       <c r="F68" s="15">
         <v>1</v>
       </c>
@@ -4749,6 +4815,7 @@
       </c>
       <c r="C69" s="25"/>
       <c r="D69" s="25"/>
+      <c r="E69" s="15"/>
       <c r="F69" s="15">
         <v>1</v>
       </c>
@@ -4791,6 +4858,7 @@
       </c>
       <c r="C70" s="25"/>
       <c r="D70" s="25"/>
+      <c r="E70" s="15"/>
       <c r="F70" s="15">
         <v>1</v>
       </c>
@@ -4833,6 +4901,7 @@
       </c>
       <c r="C71" s="25"/>
       <c r="D71" s="25"/>
+      <c r="E71" s="15"/>
       <c r="F71" s="15">
         <v>1</v>
       </c>
@@ -4875,6 +4944,7 @@
       </c>
       <c r="C72" s="25"/>
       <c r="D72" s="25"/>
+      <c r="E72" s="15"/>
       <c r="F72" s="15">
         <v>1</v>
       </c>
@@ -4917,6 +4987,7 @@
       </c>
       <c r="C73" s="25"/>
       <c r="D73" s="25"/>
+      <c r="E73" s="15"/>
       <c r="F73" s="15">
         <v>1</v>
       </c>
@@ -4959,6 +5030,7 @@
       </c>
       <c r="C74" s="25"/>
       <c r="D74" s="25"/>
+      <c r="E74" s="15"/>
       <c r="F74" s="15">
         <v>1</v>
       </c>
@@ -5001,6 +5073,7 @@
       </c>
       <c r="C75" s="25"/>
       <c r="D75" s="25"/>
+      <c r="E75" s="15"/>
       <c r="F75" s="15">
         <v>1</v>
       </c>
@@ -5043,6 +5116,7 @@
       </c>
       <c r="C76" s="25"/>
       <c r="D76" s="25"/>
+      <c r="E76" s="15"/>
       <c r="F76" s="15">
         <v>1</v>
       </c>
@@ -5085,6 +5159,7 @@
       </c>
       <c r="C77" s="25"/>
       <c r="D77" s="25"/>
+      <c r="E77" s="15"/>
       <c r="F77" s="15">
         <v>1</v>
       </c>
@@ -5127,6 +5202,7 @@
       </c>
       <c r="C78" s="25"/>
       <c r="D78" s="25"/>
+      <c r="E78" s="15"/>
       <c r="F78" s="15">
         <v>1</v>
       </c>
@@ -5169,6 +5245,7 @@
       </c>
       <c r="C79" s="25"/>
       <c r="D79" s="25"/>
+      <c r="E79" s="15"/>
       <c r="F79" s="15">
         <v>1</v>
       </c>
@@ -5211,6 +5288,7 @@
       </c>
       <c r="C80" s="25"/>
       <c r="D80" s="25"/>
+      <c r="E80" s="15"/>
       <c r="F80" s="15">
         <v>1</v>
       </c>
@@ -5253,6 +5331,7 @@
       </c>
       <c r="C81" s="25"/>
       <c r="D81" s="25"/>
+      <c r="E81" s="15"/>
       <c r="F81" s="15">
         <v>1</v>
       </c>
@@ -5295,6 +5374,7 @@
       </c>
       <c r="C82" s="25"/>
       <c r="D82" s="25"/>
+      <c r="E82" s="15"/>
       <c r="F82" s="15">
         <v>1</v>
       </c>
@@ -5337,6 +5417,7 @@
       </c>
       <c r="C83" s="25"/>
       <c r="D83" s="25"/>
+      <c r="E83" s="15"/>
       <c r="F83" s="15">
         <v>1</v>
       </c>
@@ -5379,6 +5460,7 @@
       </c>
       <c r="C84" s="25"/>
       <c r="D84" s="25"/>
+      <c r="E84" s="15"/>
       <c r="F84" s="15">
         <v>1</v>
       </c>
@@ -5421,6 +5503,7 @@
       </c>
       <c r="C85" s="25"/>
       <c r="D85" s="25"/>
+      <c r="E85" s="15"/>
       <c r="F85" s="15">
         <v>1</v>
       </c>
@@ -5463,6 +5546,7 @@
       </c>
       <c r="C86" s="25"/>
       <c r="D86" s="25"/>
+      <c r="E86" s="15"/>
       <c r="F86" s="15">
         <v>1</v>
       </c>
@@ -5505,6 +5589,7 @@
       </c>
       <c r="C87" s="25"/>
       <c r="D87" s="25"/>
+      <c r="E87" s="15"/>
       <c r="F87" s="15">
         <v>1</v>
       </c>
@@ -5547,6 +5632,7 @@
       </c>
       <c r="C88" s="25"/>
       <c r="D88" s="25"/>
+      <c r="E88" s="15"/>
       <c r="F88" s="15">
         <v>1</v>
       </c>
@@ -5589,6 +5675,7 @@
       </c>
       <c r="C89" s="25"/>
       <c r="D89" s="25"/>
+      <c r="E89" s="15"/>
       <c r="F89" s="15">
         <v>1</v>
       </c>
@@ -5631,6 +5718,7 @@
       </c>
       <c r="C90" s="25"/>
       <c r="D90" s="25"/>
+      <c r="E90" s="15"/>
       <c r="F90" s="15">
         <v>1</v>
       </c>
@@ -5673,6 +5761,7 @@
       </c>
       <c r="C91" s="25"/>
       <c r="D91" s="25"/>
+      <c r="E91" s="15"/>
       <c r="F91" s="15">
         <v>1</v>
       </c>
@@ -5715,6 +5804,7 @@
       </c>
       <c r="C92" s="25"/>
       <c r="D92" s="25"/>
+      <c r="E92" s="15"/>
       <c r="F92" s="15">
         <v>1</v>
       </c>
@@ -5757,6 +5847,7 @@
       </c>
       <c r="C93" s="25"/>
       <c r="D93" s="25"/>
+      <c r="E93" s="15"/>
       <c r="F93" s="15">
         <v>1</v>
       </c>
@@ -5799,6 +5890,7 @@
       </c>
       <c r="C94" s="25"/>
       <c r="D94" s="25"/>
+      <c r="E94" s="15"/>
       <c r="F94" s="15">
         <v>1</v>
       </c>
@@ -5841,6 +5933,7 @@
       </c>
       <c r="C95" s="25"/>
       <c r="D95" s="25"/>
+      <c r="E95" s="15"/>
       <c r="F95" s="15">
         <v>1</v>
       </c>
@@ -5883,6 +5976,7 @@
       </c>
       <c r="C96" s="25"/>
       <c r="D96" s="25"/>
+      <c r="E96" s="15"/>
       <c r="F96" s="15">
         <v>1</v>
       </c>
@@ -5925,6 +6019,7 @@
       </c>
       <c r="C97" s="25"/>
       <c r="D97" s="25"/>
+      <c r="E97" s="15"/>
       <c r="F97" s="15">
         <v>1</v>
       </c>
@@ -5967,6 +6062,7 @@
       </c>
       <c r="C98" s="25"/>
       <c r="D98" s="25"/>
+      <c r="E98" s="15"/>
       <c r="F98" s="15">
         <v>1</v>
       </c>
@@ -6009,6 +6105,7 @@
       </c>
       <c r="C99" s="25"/>
       <c r="D99" s="25"/>
+      <c r="E99" s="15"/>
       <c r="F99" s="15">
         <v>1</v>
       </c>
@@ -6051,6 +6148,7 @@
       </c>
       <c r="C100" s="25"/>
       <c r="D100" s="25"/>
+      <c r="E100" s="15"/>
       <c r="F100" s="15">
         <v>1</v>
       </c>
@@ -6093,6 +6191,7 @@
       </c>
       <c r="C101" s="25"/>
       <c r="D101" s="25"/>
+      <c r="E101" s="15"/>
       <c r="F101" s="15">
         <v>1</v>
       </c>
@@ -6135,6 +6234,7 @@
       </c>
       <c r="C102" s="25"/>
       <c r="D102" s="25"/>
+      <c r="E102" s="15"/>
       <c r="F102" s="15">
         <v>1</v>
       </c>
@@ -6177,6 +6277,7 @@
       </c>
       <c r="C103" s="25"/>
       <c r="D103" s="25"/>
+      <c r="E103" s="15"/>
       <c r="F103" s="15">
         <v>1</v>
       </c>
@@ -6219,6 +6320,7 @@
       </c>
       <c r="C104" s="25"/>
       <c r="D104" s="25"/>
+      <c r="E104" s="15"/>
       <c r="F104" s="15">
         <v>1</v>
       </c>
@@ -6261,6 +6363,7 @@
       </c>
       <c r="C105" s="25"/>
       <c r="D105" s="25"/>
+      <c r="E105" s="15"/>
       <c r="F105" s="15">
         <v>1</v>
       </c>
@@ -6303,6 +6406,7 @@
       </c>
       <c r="C106" s="25"/>
       <c r="D106" s="25"/>
+      <c r="E106" s="15"/>
       <c r="F106" s="15">
         <v>1</v>
       </c>
@@ -6345,6 +6449,7 @@
       </c>
       <c r="C107" s="25"/>
       <c r="D107" s="25"/>
+      <c r="E107" s="15"/>
       <c r="F107" s="15">
         <v>1</v>
       </c>
@@ -6387,6 +6492,7 @@
       </c>
       <c r="C108" s="25"/>
       <c r="D108" s="25"/>
+      <c r="E108" s="15"/>
       <c r="F108" s="15">
         <v>1</v>
       </c>
@@ -6429,6 +6535,7 @@
       </c>
       <c r="C109" s="25"/>
       <c r="D109" s="25"/>
+      <c r="E109" s="15"/>
       <c r="F109" s="15">
         <v>1</v>
       </c>
@@ -6471,6 +6578,7 @@
       </c>
       <c r="C110" s="25"/>
       <c r="D110" s="25"/>
+      <c r="E110" s="15"/>
       <c r="F110" s="15">
         <v>1</v>
       </c>
@@ -6513,6 +6621,7 @@
       </c>
       <c r="C111" s="25"/>
       <c r="D111" s="25"/>
+      <c r="E111" s="15"/>
       <c r="F111" s="15">
         <v>1</v>
       </c>
@@ -6555,6 +6664,7 @@
       </c>
       <c r="C112" s="25"/>
       <c r="D112" s="25"/>
+      <c r="E112" s="15"/>
       <c r="F112" s="15">
         <v>1</v>
       </c>
@@ -6597,6 +6707,7 @@
       </c>
       <c r="C113" s="25"/>
       <c r="D113" s="25"/>
+      <c r="E113" s="15"/>
       <c r="F113" s="15">
         <v>1</v>
       </c>
@@ -6639,6 +6750,7 @@
       </c>
       <c r="C114" s="25"/>
       <c r="D114" s="25"/>
+      <c r="E114" s="15"/>
       <c r="F114" s="15">
         <v>1</v>
       </c>
@@ -6681,6 +6793,7 @@
       </c>
       <c r="C115" s="25"/>
       <c r="D115" s="25"/>
+      <c r="E115" s="15"/>
       <c r="F115" s="15">
         <v>1</v>
       </c>
@@ -6723,6 +6836,7 @@
       </c>
       <c r="C116" s="25"/>
       <c r="D116" s="25"/>
+      <c r="E116" s="15"/>
       <c r="F116" s="15">
         <v>1</v>
       </c>
@@ -6765,6 +6879,7 @@
       </c>
       <c r="C117" s="25"/>
       <c r="D117" s="25"/>
+      <c r="E117" s="15"/>
       <c r="F117" s="15">
         <v>1</v>
       </c>
@@ -6807,6 +6922,7 @@
       </c>
       <c r="C118" s="25"/>
       <c r="D118" s="25"/>
+      <c r="E118" s="15"/>
       <c r="F118" s="15">
         <v>1</v>
       </c>
@@ -6849,6 +6965,7 @@
       </c>
       <c r="C119" s="25"/>
       <c r="D119" s="25"/>
+      <c r="E119" s="15"/>
       <c r="F119" s="15">
         <v>1</v>
       </c>
@@ -6891,6 +7008,7 @@
       </c>
       <c r="C120" s="25"/>
       <c r="D120" s="25"/>
+      <c r="E120" s="15"/>
       <c r="F120" s="15">
         <v>1</v>
       </c>
@@ -6933,6 +7051,7 @@
       </c>
       <c r="C121" s="25"/>
       <c r="D121" s="25"/>
+      <c r="E121" s="15"/>
       <c r="F121" s="15">
         <v>1</v>
       </c>
@@ -6975,6 +7094,7 @@
       </c>
       <c r="C122" s="25"/>
       <c r="D122" s="25"/>
+      <c r="E122" s="15"/>
       <c r="F122" s="15">
         <v>1</v>
       </c>
@@ -7017,6 +7137,7 @@
       </c>
       <c r="C123" s="25"/>
       <c r="D123" s="25"/>
+      <c r="E123" s="15"/>
       <c r="F123" s="15">
         <v>1</v>
       </c>
@@ -7059,6 +7180,7 @@
       </c>
       <c r="C124" s="25"/>
       <c r="D124" s="25"/>
+      <c r="E124" s="15"/>
       <c r="F124" s="15">
         <v>1</v>
       </c>
@@ -7101,6 +7223,7 @@
       </c>
       <c r="C125" s="25"/>
       <c r="D125" s="25"/>
+      <c r="E125" s="15"/>
       <c r="F125" s="15">
         <v>1</v>
       </c>
@@ -7143,6 +7266,7 @@
       </c>
       <c r="C126" s="25"/>
       <c r="D126" s="25"/>
+      <c r="E126" s="15"/>
       <c r="F126" s="15">
         <v>1</v>
       </c>
@@ -7185,6 +7309,7 @@
       </c>
       <c r="C127" s="25"/>
       <c r="D127" s="25"/>
+      <c r="E127" s="15"/>
       <c r="F127" s="15">
         <v>1</v>
       </c>
@@ -7227,6 +7352,7 @@
       </c>
       <c r="C128" s="25"/>
       <c r="D128" s="25"/>
+      <c r="E128" s="15"/>
       <c r="F128" s="15">
         <v>1</v>
       </c>
@@ -7269,6 +7395,7 @@
       </c>
       <c r="C129" s="25"/>
       <c r="D129" s="25"/>
+      <c r="E129" s="15"/>
       <c r="F129" s="15">
         <v>1</v>
       </c>
@@ -7311,6 +7438,7 @@
       </c>
       <c r="C130" s="25"/>
       <c r="D130" s="25"/>
+      <c r="E130" s="15"/>
       <c r="F130" s="15">
         <v>1</v>
       </c>
@@ -7353,6 +7481,7 @@
       </c>
       <c r="C131" s="25"/>
       <c r="D131" s="25"/>
+      <c r="E131" s="15"/>
       <c r="F131" s="15">
         <v>1</v>
       </c>
@@ -7395,6 +7524,7 @@
       </c>
       <c r="C132" s="25"/>
       <c r="D132" s="25"/>
+      <c r="E132" s="15"/>
       <c r="F132" s="15">
         <v>1</v>
       </c>
@@ -7437,6 +7567,7 @@
       </c>
       <c r="C133" s="25"/>
       <c r="D133" s="25"/>
+      <c r="E133" s="15"/>
       <c r="F133" s="15">
         <v>1</v>
       </c>
@@ -7479,6 +7610,7 @@
       </c>
       <c r="C134" s="25"/>
       <c r="D134" s="25"/>
+      <c r="E134" s="15"/>
       <c r="F134" s="15">
         <v>1</v>
       </c>
@@ -7521,6 +7653,7 @@
       </c>
       <c r="C135" s="25"/>
       <c r="D135" s="25"/>
+      <c r="E135" s="15"/>
       <c r="F135" s="15">
         <v>1</v>
       </c>
@@ -7563,6 +7696,7 @@
       </c>
       <c r="C136" s="25"/>
       <c r="D136" s="25"/>
+      <c r="E136" s="15"/>
       <c r="F136" s="15">
         <v>1</v>
       </c>
@@ -7605,6 +7739,7 @@
       </c>
       <c r="C137" s="25"/>
       <c r="D137" s="25"/>
+      <c r="E137" s="15"/>
       <c r="F137" s="15">
         <v>1</v>
       </c>
@@ -7647,6 +7782,7 @@
       </c>
       <c r="C138" s="25"/>
       <c r="D138" s="25"/>
+      <c r="E138" s="15"/>
       <c r="F138" s="15">
         <v>1</v>
       </c>
@@ -7689,6 +7825,7 @@
       </c>
       <c r="C139" s="25"/>
       <c r="D139" s="25"/>
+      <c r="E139" s="15"/>
       <c r="F139" s="15">
         <v>1</v>
       </c>
@@ -7731,6 +7868,7 @@
       </c>
       <c r="C140" s="25"/>
       <c r="D140" s="25"/>
+      <c r="E140" s="15"/>
       <c r="F140" s="15">
         <v>1</v>
       </c>
@@ -7773,6 +7911,7 @@
       </c>
       <c r="C141" s="25"/>
       <c r="D141" s="25"/>
+      <c r="E141" s="15"/>
       <c r="F141" s="15">
         <v>1</v>
       </c>
@@ -7815,6 +7954,7 @@
       </c>
       <c r="C142" s="25"/>
       <c r="D142" s="25"/>
+      <c r="E142" s="15"/>
       <c r="F142" s="15">
         <v>1</v>
       </c>
@@ -7857,6 +7997,7 @@
       </c>
       <c r="C143" s="25"/>
       <c r="D143" s="25"/>
+      <c r="E143" s="15"/>
       <c r="F143" s="15">
         <v>1</v>
       </c>
@@ -7899,6 +8040,7 @@
       </c>
       <c r="C144" s="25"/>
       <c r="D144" s="25"/>
+      <c r="E144" s="15"/>
       <c r="F144" s="15">
         <v>1</v>
       </c>
@@ -7941,6 +8083,7 @@
       </c>
       <c r="C145" s="25"/>
       <c r="D145" s="25"/>
+      <c r="E145" s="15"/>
       <c r="F145" s="15">
         <v>1</v>
       </c>
@@ -7983,6 +8126,7 @@
       </c>
       <c r="C146" s="25"/>
       <c r="D146" s="25"/>
+      <c r="E146" s="15"/>
       <c r="F146" s="15">
         <v>1</v>
       </c>
@@ -8025,6 +8169,7 @@
       </c>
       <c r="C147" s="25"/>
       <c r="D147" s="25"/>
+      <c r="E147" s="15"/>
       <c r="F147" s="15">
         <v>1</v>
       </c>
@@ -8067,6 +8212,7 @@
       </c>
       <c r="C148" s="25"/>
       <c r="D148" s="25"/>
+      <c r="E148" s="15"/>
       <c r="F148" s="15">
         <v>1</v>
       </c>
@@ -8109,6 +8255,7 @@
       </c>
       <c r="C149" s="25"/>
       <c r="D149" s="25"/>
+      <c r="E149" s="15"/>
       <c r="F149" s="15">
         <v>1</v>
       </c>
@@ -8151,6 +8298,7 @@
       </c>
       <c r="C150" s="25"/>
       <c r="D150" s="25"/>
+      <c r="E150" s="15"/>
       <c r="F150" s="15">
         <v>1</v>
       </c>
@@ -8193,6 +8341,7 @@
       </c>
       <c r="C151" s="25"/>
       <c r="D151" s="25"/>
+      <c r="E151" s="15"/>
       <c r="F151" s="15">
         <v>1</v>
       </c>
@@ -8235,6 +8384,7 @@
       </c>
       <c r="C152" s="25"/>
       <c r="D152" s="25"/>
+      <c r="E152" s="15"/>
       <c r="F152" s="15">
         <v>1</v>
       </c>
@@ -8277,6 +8427,7 @@
       </c>
       <c r="C153" s="25"/>
       <c r="D153" s="25"/>
+      <c r="E153" s="15"/>
       <c r="F153" s="15">
         <v>1</v>
       </c>
@@ -8319,6 +8470,7 @@
       </c>
       <c r="C154" s="25"/>
       <c r="D154" s="25"/>
+      <c r="E154" s="15"/>
       <c r="F154" s="15">
         <v>1</v>
       </c>
@@ -8361,6 +8513,7 @@
       </c>
       <c r="C155" s="25"/>
       <c r="D155" s="25"/>
+      <c r="E155" s="15"/>
       <c r="F155" s="15">
         <v>1</v>
       </c>
@@ -8403,6 +8556,7 @@
       </c>
       <c r="C156" s="25"/>
       <c r="D156" s="25"/>
+      <c r="E156" s="15"/>
       <c r="F156" s="15">
         <v>1</v>
       </c>
@@ -8445,6 +8599,7 @@
       </c>
       <c r="C157" s="25"/>
       <c r="D157" s="25"/>
+      <c r="E157" s="15"/>
       <c r="F157" s="15">
         <v>1</v>
       </c>
@@ -8487,6 +8642,7 @@
       </c>
       <c r="C158" s="25"/>
       <c r="D158" s="25"/>
+      <c r="E158" s="15"/>
       <c r="F158" s="15">
         <v>1</v>
       </c>
@@ -8529,6 +8685,7 @@
       </c>
       <c r="C159" s="25"/>
       <c r="D159" s="25"/>
+      <c r="E159" s="15"/>
       <c r="F159" s="15">
         <v>1</v>
       </c>
@@ -8571,6 +8728,7 @@
       </c>
       <c r="C160" s="25"/>
       <c r="D160" s="25"/>
+      <c r="E160" s="15"/>
       <c r="F160" s="15">
         <v>1</v>
       </c>
@@ -8613,6 +8771,7 @@
       </c>
       <c r="C161" s="25"/>
       <c r="D161" s="25"/>
+      <c r="E161" s="15"/>
       <c r="F161" s="15">
         <v>1</v>
       </c>
@@ -8655,6 +8814,7 @@
       </c>
       <c r="C162" s="25"/>
       <c r="D162" s="25"/>
+      <c r="E162" s="15"/>
       <c r="F162" s="15">
         <v>1</v>
       </c>
@@ -8697,6 +8857,7 @@
       </c>
       <c r="C163" s="25"/>
       <c r="D163" s="25"/>
+      <c r="E163" s="15"/>
       <c r="F163" s="15">
         <v>1</v>
       </c>
@@ -8739,6 +8900,7 @@
       </c>
       <c r="C164" s="25"/>
       <c r="D164" s="25"/>
+      <c r="E164" s="15"/>
       <c r="F164" s="15">
         <v>1</v>
       </c>
@@ -8781,6 +8943,7 @@
       </c>
       <c r="C165" s="25"/>
       <c r="D165" s="25"/>
+      <c r="E165" s="15"/>
       <c r="F165" s="15">
         <v>1</v>
       </c>
@@ -8823,6 +8986,7 @@
       </c>
       <c r="C166" s="25"/>
       <c r="D166" s="25"/>
+      <c r="E166" s="15"/>
       <c r="F166" s="15">
         <v>1</v>
       </c>
@@ -8865,6 +9029,7 @@
       </c>
       <c r="C167" s="25"/>
       <c r="D167" s="25"/>
+      <c r="E167" s="15"/>
       <c r="F167" s="15">
         <v>1</v>
       </c>
@@ -8907,6 +9072,7 @@
       </c>
       <c r="C168" s="25"/>
       <c r="D168" s="25"/>
+      <c r="E168" s="15"/>
       <c r="F168" s="15">
         <v>1</v>
       </c>
@@ -8949,6 +9115,7 @@
       </c>
       <c r="C169" s="25"/>
       <c r="D169" s="25"/>
+      <c r="E169" s="15"/>
       <c r="F169" s="15">
         <v>1</v>
       </c>
@@ -8991,6 +9158,7 @@
       </c>
       <c r="C170" s="25"/>
       <c r="D170" s="25"/>
+      <c r="E170" s="15"/>
       <c r="F170" s="15">
         <v>1</v>
       </c>
@@ -9033,6 +9201,7 @@
       </c>
       <c r="C171" s="25"/>
       <c r="D171" s="25"/>
+      <c r="E171" s="15"/>
       <c r="F171" s="15">
         <v>1</v>
       </c>
@@ -9075,6 +9244,7 @@
       </c>
       <c r="C172" s="25"/>
       <c r="D172" s="25"/>
+      <c r="E172" s="15"/>
       <c r="F172" s="15">
         <v>1</v>
       </c>
@@ -9117,6 +9287,7 @@
       </c>
       <c r="C173" s="25"/>
       <c r="D173" s="25"/>
+      <c r="E173" s="15"/>
       <c r="F173" s="15">
         <v>1</v>
       </c>
@@ -9159,6 +9330,7 @@
       </c>
       <c r="C174" s="25"/>
       <c r="D174" s="25"/>
+      <c r="E174" s="15"/>
       <c r="F174" s="15">
         <v>1</v>
       </c>
@@ -9201,6 +9373,7 @@
       </c>
       <c r="C175" s="25"/>
       <c r="D175" s="25"/>
+      <c r="E175" s="15"/>
       <c r="F175" s="15">
         <v>1</v>
       </c>
@@ -9243,6 +9416,7 @@
       </c>
       <c r="C176" s="25"/>
       <c r="D176" s="25"/>
+      <c r="E176" s="15"/>
       <c r="F176" s="15">
         <v>1</v>
       </c>
@@ -9285,6 +9459,7 @@
       </c>
       <c r="C177" s="25"/>
       <c r="D177" s="25"/>
+      <c r="E177" s="15"/>
       <c r="F177" s="15">
         <v>1</v>
       </c>
@@ -9327,6 +9502,7 @@
       </c>
       <c r="C178" s="25"/>
       <c r="D178" s="25"/>
+      <c r="E178" s="15"/>
       <c r="F178" s="15">
         <v>1</v>
       </c>
@@ -9369,6 +9545,7 @@
       </c>
       <c r="C179" s="25"/>
       <c r="D179" s="25"/>
+      <c r="E179" s="15"/>
       <c r="F179" s="15">
         <v>1</v>
       </c>
@@ -9411,6 +9588,7 @@
       </c>
       <c r="C180" s="25"/>
       <c r="D180" s="25"/>
+      <c r="E180" s="15"/>
       <c r="F180" s="15">
         <v>1</v>
       </c>
@@ -9453,6 +9631,7 @@
       </c>
       <c r="C181" s="25"/>
       <c r="D181" s="25"/>
+      <c r="E181" s="15"/>
       <c r="F181" s="15">
         <v>1</v>
       </c>
@@ -9495,6 +9674,7 @@
       </c>
       <c r="C182" s="25"/>
       <c r="D182" s="25"/>
+      <c r="E182" s="15"/>
       <c r="F182" s="15">
         <v>1</v>
       </c>
@@ -9537,6 +9717,7 @@
       </c>
       <c r="C183" s="25"/>
       <c r="D183" s="25"/>
+      <c r="E183" s="15"/>
       <c r="F183" s="15">
         <v>1</v>
       </c>
@@ -9579,6 +9760,7 @@
       </c>
       <c r="C184" s="25"/>
       <c r="D184" s="25"/>
+      <c r="E184" s="15"/>
       <c r="F184" s="15">
         <v>1</v>
       </c>
@@ -9621,6 +9803,7 @@
       </c>
       <c r="C185" s="25"/>
       <c r="D185" s="25"/>
+      <c r="E185" s="15"/>
       <c r="F185" s="15">
         <v>1</v>
       </c>
@@ -9663,6 +9846,7 @@
       </c>
       <c r="C186" s="25"/>
       <c r="D186" s="25"/>
+      <c r="E186" s="15"/>
       <c r="F186" s="15">
         <v>1</v>
       </c>
@@ -9705,6 +9889,7 @@
       </c>
       <c r="C187" s="25"/>
       <c r="D187" s="25"/>
+      <c r="E187" s="15"/>
       <c r="F187" s="15">
         <v>1</v>
       </c>
@@ -9747,6 +9932,7 @@
       </c>
       <c r="C188" s="25"/>
       <c r="D188" s="25"/>
+      <c r="E188" s="15"/>
       <c r="F188" s="15">
         <v>1</v>
       </c>
@@ -9789,6 +9975,7 @@
       </c>
       <c r="C189" s="25"/>
       <c r="D189" s="25"/>
+      <c r="E189" s="15"/>
       <c r="F189" s="15">
         <v>1</v>
       </c>
@@ -9831,6 +10018,7 @@
       </c>
       <c r="C190" s="25"/>
       <c r="D190" s="25"/>
+      <c r="E190" s="15"/>
       <c r="F190" s="15">
         <v>1</v>
       </c>
@@ -9873,6 +10061,7 @@
       </c>
       <c r="C191" s="25"/>
       <c r="D191" s="25"/>
+      <c r="E191" s="15"/>
       <c r="F191" s="15">
         <v>1</v>
       </c>
@@ -9915,6 +10104,7 @@
       </c>
       <c r="C192" s="25"/>
       <c r="D192" s="25"/>
+      <c r="E192" s="15"/>
       <c r="F192" s="15">
         <v>1</v>
       </c>
@@ -9957,6 +10147,7 @@
       </c>
       <c r="C193" s="25"/>
       <c r="D193" s="25"/>
+      <c r="E193" s="15"/>
       <c r="F193" s="15">
         <v>1</v>
       </c>
@@ -9999,6 +10190,7 @@
       </c>
       <c r="C194" s="25"/>
       <c r="D194" s="25"/>
+      <c r="E194" s="15"/>
       <c r="F194" s="15">
         <v>1</v>
       </c>
@@ -10041,6 +10233,7 @@
       </c>
       <c r="C195" s="25"/>
       <c r="D195" s="25"/>
+      <c r="E195" s="15"/>
       <c r="F195" s="15">
         <v>1</v>
       </c>
@@ -10083,6 +10276,7 @@
       </c>
       <c r="C196" s="25"/>
       <c r="D196" s="25"/>
+      <c r="E196" s="15"/>
       <c r="F196" s="15">
         <v>1</v>
       </c>
@@ -10125,6 +10319,7 @@
       </c>
       <c r="C197" s="25"/>
       <c r="D197" s="25"/>
+      <c r="E197" s="15"/>
       <c r="F197" s="15">
         <v>1</v>
       </c>
@@ -10167,6 +10362,7 @@
       </c>
       <c r="C198" s="25"/>
       <c r="D198" s="25"/>
+      <c r="E198" s="15"/>
       <c r="F198" s="15">
         <v>1</v>
       </c>
@@ -10209,6 +10405,7 @@
       </c>
       <c r="C199" s="25"/>
       <c r="D199" s="25"/>
+      <c r="E199" s="15"/>
       <c r="F199" s="15">
         <v>1</v>
       </c>
@@ -10251,6 +10448,7 @@
       </c>
       <c r="C200" s="25"/>
       <c r="D200" s="25"/>
+      <c r="E200" s="15"/>
       <c r="F200" s="15">
         <v>1</v>
       </c>
@@ -10293,6 +10491,7 @@
       </c>
       <c r="C201" s="25"/>
       <c r="D201" s="25"/>
+      <c r="E201" s="15"/>
       <c r="F201" s="15">
         <v>1</v>
       </c>
@@ -10335,6 +10534,7 @@
       </c>
       <c r="C202" s="25"/>
       <c r="D202" s="25"/>
+      <c r="E202" s="15"/>
       <c r="F202" s="15">
         <v>1</v>
       </c>
@@ -10377,6 +10577,7 @@
       </c>
       <c r="C203" s="25"/>
       <c r="D203" s="25"/>
+      <c r="E203" s="15"/>
       <c r="F203" s="15">
         <v>1</v>
       </c>
@@ -10419,6 +10620,7 @@
       </c>
       <c r="C204" s="25"/>
       <c r="D204" s="25"/>
+      <c r="E204" s="15"/>
       <c r="F204" s="15">
         <v>1</v>
       </c>
@@ -10461,6 +10663,7 @@
       </c>
       <c r="C205" s="25"/>
       <c r="D205" s="25"/>
+      <c r="E205" s="15"/>
       <c r="F205" s="15">
         <v>1</v>
       </c>
@@ -10503,6 +10706,7 @@
       </c>
       <c r="C206" s="25"/>
       <c r="D206" s="25"/>
+      <c r="E206" s="15"/>
       <c r="F206" s="15">
         <v>1</v>
       </c>
@@ -10545,6 +10749,7 @@
       </c>
       <c r="C207" s="25"/>
       <c r="D207" s="25"/>
+      <c r="E207" s="15"/>
       <c r="F207" s="15">
         <v>1</v>
       </c>
@@ -10587,6 +10792,7 @@
       </c>
       <c r="C208" s="25"/>
       <c r="D208" s="25"/>
+      <c r="E208" s="15"/>
       <c r="F208" s="15">
         <v>1</v>
       </c>
@@ -10629,6 +10835,7 @@
       </c>
       <c r="C209" s="25"/>
       <c r="D209" s="25"/>
+      <c r="E209" s="15"/>
       <c r="F209" s="15">
         <v>1</v>
       </c>
@@ -10671,6 +10878,7 @@
       </c>
       <c r="C210" s="25"/>
       <c r="D210" s="25"/>
+      <c r="E210" s="15"/>
       <c r="F210" s="15">
         <v>1</v>
       </c>
@@ -10713,6 +10921,7 @@
       </c>
       <c r="C211" s="25"/>
       <c r="D211" s="25"/>
+      <c r="E211" s="15"/>
       <c r="F211" s="15">
         <v>1</v>
       </c>
@@ -10755,6 +10964,7 @@
       </c>
       <c r="C212" s="25"/>
       <c r="D212" s="25"/>
+      <c r="E212" s="15"/>
       <c r="F212" s="15">
         <v>1</v>
       </c>
@@ -10797,6 +11007,7 @@
       </c>
       <c r="C213" s="25"/>
       <c r="D213" s="25"/>
+      <c r="E213" s="15"/>
       <c r="F213" s="15">
         <v>1</v>
       </c>
@@ -10839,6 +11050,7 @@
       </c>
       <c r="C214" s="25"/>
       <c r="D214" s="25"/>
+      <c r="E214" s="15"/>
       <c r="F214" s="15">
         <v>1</v>
       </c>
@@ -10881,6 +11093,7 @@
       </c>
       <c r="C215" s="25"/>
       <c r="D215" s="25"/>
+      <c r="E215" s="15"/>
       <c r="F215" s="15">
         <v>1</v>
       </c>
@@ -10923,6 +11136,7 @@
       </c>
       <c r="C216" s="25"/>
       <c r="D216" s="25"/>
+      <c r="E216" s="15"/>
       <c r="F216" s="15">
         <v>1</v>
       </c>
@@ -10965,6 +11179,7 @@
       </c>
       <c r="C217" s="25"/>
       <c r="D217" s="25"/>
+      <c r="E217" s="15"/>
       <c r="F217" s="15">
         <v>1</v>
       </c>
@@ -11007,6 +11222,7 @@
       </c>
       <c r="C218" s="25"/>
       <c r="D218" s="25"/>
+      <c r="E218" s="15"/>
       <c r="F218" s="15">
         <v>1</v>
       </c>
@@ -11049,6 +11265,7 @@
       </c>
       <c r="C219" s="25"/>
       <c r="D219" s="25"/>
+      <c r="E219" s="15"/>
       <c r="F219" s="15">
         <v>1</v>
       </c>
@@ -11091,6 +11308,7 @@
       </c>
       <c r="C220" s="25"/>
       <c r="D220" s="25"/>
+      <c r="E220" s="15"/>
       <c r="F220" s="15">
         <v>1</v>
       </c>
@@ -11133,6 +11351,7 @@
       </c>
       <c r="C221" s="25"/>
       <c r="D221" s="25"/>
+      <c r="E221" s="15"/>
       <c r="F221" s="15">
         <v>1</v>
       </c>
@@ -11175,6 +11394,7 @@
       </c>
       <c r="C222" s="25"/>
       <c r="D222" s="25"/>
+      <c r="E222" s="15"/>
       <c r="F222" s="15">
         <v>1</v>
       </c>
@@ -11217,6 +11437,7 @@
       </c>
       <c r="C223" s="25"/>
       <c r="D223" s="25"/>
+      <c r="E223" s="15"/>
       <c r="F223" s="15">
         <v>1</v>
       </c>
@@ -11259,6 +11480,7 @@
       </c>
       <c r="C224" s="25"/>
       <c r="D224" s="25"/>
+      <c r="E224" s="15"/>
       <c r="F224" s="15">
         <v>1</v>
       </c>
@@ -11301,6 +11523,7 @@
       </c>
       <c r="C225" s="25"/>
       <c r="D225" s="25"/>
+      <c r="E225" s="15"/>
       <c r="F225" s="15">
         <v>1</v>
       </c>
@@ -11343,6 +11566,7 @@
       </c>
       <c r="C226" s="25"/>
       <c r="D226" s="25"/>
+      <c r="E226" s="15"/>
       <c r="F226" s="15">
         <v>1</v>
       </c>
@@ -11385,6 +11609,7 @@
       </c>
       <c r="C227" s="25"/>
       <c r="D227" s="25"/>
+      <c r="E227" s="15"/>
       <c r="F227" s="15">
         <v>1</v>
       </c>
@@ -11427,6 +11652,7 @@
       </c>
       <c r="C228" s="25"/>
       <c r="D228" s="25"/>
+      <c r="E228" s="15"/>
       <c r="F228" s="15">
         <v>1</v>
       </c>
@@ -11469,6 +11695,7 @@
       </c>
       <c r="C229" s="25"/>
       <c r="D229" s="25"/>
+      <c r="E229" s="15"/>
       <c r="F229" s="15">
         <v>1</v>
       </c>
@@ -11511,6 +11738,7 @@
       </c>
       <c r="C230" s="25"/>
       <c r="D230" s="25"/>
+      <c r="E230" s="15"/>
       <c r="F230" s="15">
         <v>1</v>
       </c>
@@ -11553,6 +11781,7 @@
       </c>
       <c r="C231" s="25"/>
       <c r="D231" s="25"/>
+      <c r="E231" s="15"/>
       <c r="F231" s="15">
         <v>1</v>
       </c>
@@ -11595,6 +11824,7 @@
       </c>
       <c r="C232" s="25"/>
       <c r="D232" s="25"/>
+      <c r="E232" s="15"/>
       <c r="F232" s="15">
         <v>1</v>
       </c>
@@ -11637,6 +11867,7 @@
       </c>
       <c r="C233" s="25"/>
       <c r="D233" s="25"/>
+      <c r="E233" s="15"/>
       <c r="F233" s="15">
         <v>1</v>
       </c>
@@ -11679,6 +11910,7 @@
       </c>
       <c r="C234" s="25"/>
       <c r="D234" s="25"/>
+      <c r="E234" s="15"/>
       <c r="F234" s="15">
         <v>1</v>
       </c>
@@ -11721,6 +11953,7 @@
       </c>
       <c r="C235" s="25"/>
       <c r="D235" s="25"/>
+      <c r="E235" s="15"/>
       <c r="F235" s="15">
         <v>1</v>
       </c>
@@ -11763,6 +11996,7 @@
       </c>
       <c r="C236" s="25"/>
       <c r="D236" s="25"/>
+      <c r="E236" s="15"/>
       <c r="F236" s="15">
         <v>1</v>
       </c>
@@ -11805,6 +12039,7 @@
       </c>
       <c r="C237" s="25"/>
       <c r="D237" s="25"/>
+      <c r="E237" s="15"/>
       <c r="F237" s="15">
         <v>1</v>
       </c>
@@ -11847,6 +12082,7 @@
       </c>
       <c r="C238" s="25"/>
       <c r="D238" s="25"/>
+      <c r="E238" s="15"/>
       <c r="F238" s="15">
         <v>1</v>
       </c>
@@ -11889,6 +12125,7 @@
       </c>
       <c r="C239" s="25"/>
       <c r="D239" s="25"/>
+      <c r="E239" s="15"/>
       <c r="F239" s="15">
         <v>1</v>
       </c>
@@ -11931,6 +12168,7 @@
       </c>
       <c r="C240" s="25"/>
       <c r="D240" s="25"/>
+      <c r="E240" s="15"/>
       <c r="F240" s="15">
         <v>1</v>
       </c>
@@ -11973,6 +12211,7 @@
       </c>
       <c r="C241" s="25"/>
       <c r="D241" s="25"/>
+      <c r="E241" s="15"/>
       <c r="F241" s="15">
         <v>1</v>
       </c>
@@ -12015,6 +12254,7 @@
       </c>
       <c r="C242" s="25"/>
       <c r="D242" s="25"/>
+      <c r="E242" s="15"/>
       <c r="F242" s="15">
         <v>1</v>
       </c>
@@ -12057,6 +12297,7 @@
       </c>
       <c r="C243" s="25"/>
       <c r="D243" s="25"/>
+      <c r="E243" s="15"/>
       <c r="F243" s="15">
         <v>1</v>
       </c>
@@ -12099,6 +12340,7 @@
       </c>
       <c r="C244" s="25"/>
       <c r="D244" s="25"/>
+      <c r="E244" s="15"/>
       <c r="F244" s="15">
         <v>1</v>
       </c>
@@ -12141,6 +12383,7 @@
       </c>
       <c r="C245" s="25"/>
       <c r="D245" s="25"/>
+      <c r="E245" s="15"/>
       <c r="F245" s="15">
         <v>1</v>
       </c>
@@ -12183,6 +12426,7 @@
       </c>
       <c r="C246" s="25"/>
       <c r="D246" s="25"/>
+      <c r="E246" s="15"/>
       <c r="F246" s="15">
         <v>1</v>
       </c>
@@ -12225,6 +12469,7 @@
       </c>
       <c r="C247" s="25"/>
       <c r="D247" s="25"/>
+      <c r="E247" s="15"/>
       <c r="F247" s="15">
         <v>1</v>
       </c>
@@ -12267,6 +12512,7 @@
       </c>
       <c r="C248" s="25"/>
       <c r="D248" s="25"/>
+      <c r="E248" s="15"/>
       <c r="F248" s="15">
         <v>1</v>
       </c>
@@ -12309,6 +12555,7 @@
       </c>
       <c r="C249" s="25"/>
       <c r="D249" s="25"/>
+      <c r="E249" s="15"/>
       <c r="F249" s="15">
         <v>1</v>
       </c>
@@ -12351,6 +12598,7 @@
       </c>
       <c r="C250" s="25"/>
       <c r="D250" s="25"/>
+      <c r="E250" s="15"/>
       <c r="F250" s="15">
         <v>1</v>
       </c>
@@ -12393,6 +12641,7 @@
       </c>
       <c r="C251" s="25"/>
       <c r="D251" s="25"/>
+      <c r="E251" s="15"/>
       <c r="F251" s="15">
         <v>1</v>
       </c>
@@ -12435,6 +12684,7 @@
       </c>
       <c r="C252" s="25"/>
       <c r="D252" s="25"/>
+      <c r="E252" s="15"/>
       <c r="F252" s="15">
         <v>1</v>
       </c>
@@ -12477,6 +12727,7 @@
       </c>
       <c r="C253" s="25"/>
       <c r="D253" s="25"/>
+      <c r="E253" s="15"/>
       <c r="F253" s="15">
         <v>1</v>
       </c>
@@ -12519,6 +12770,7 @@
       </c>
       <c r="C254" s="25"/>
       <c r="D254" s="25"/>
+      <c r="E254" s="15"/>
       <c r="F254" s="15">
         <v>1</v>
       </c>
@@ -12561,6 +12813,7 @@
       </c>
       <c r="C255" s="25"/>
       <c r="D255" s="25"/>
+      <c r="E255" s="15"/>
       <c r="F255" s="15">
         <v>1</v>
       </c>
@@ -12603,6 +12856,7 @@
       </c>
       <c r="C256" s="25"/>
       <c r="D256" s="25"/>
+      <c r="E256" s="15"/>
       <c r="F256" s="15">
         <v>1</v>
       </c>
@@ -12645,6 +12899,7 @@
       </c>
       <c r="C257" s="25"/>
       <c r="D257" s="25"/>
+      <c r="E257" s="15"/>
       <c r="F257" s="15">
         <v>1</v>
       </c>
@@ -12687,6 +12942,7 @@
       </c>
       <c r="C258" s="25"/>
       <c r="D258" s="25"/>
+      <c r="E258" s="15"/>
       <c r="F258" s="15">
         <v>1</v>
       </c>
@@ -12729,6 +12985,7 @@
       </c>
       <c r="C259" s="25"/>
       <c r="D259" s="25"/>
+      <c r="E259" s="15"/>
       <c r="F259" s="15">
         <v>1</v>
       </c>
@@ -12771,6 +13028,7 @@
       </c>
       <c r="C260" s="25"/>
       <c r="D260" s="25"/>
+      <c r="E260" s="15"/>
       <c r="F260" s="15">
         <v>1</v>
       </c>
@@ -12813,6 +13071,7 @@
       </c>
       <c r="C261" s="25"/>
       <c r="D261" s="25"/>
+      <c r="E261" s="15"/>
       <c r="F261" s="15">
         <v>1</v>
       </c>
@@ -12855,6 +13114,7 @@
       </c>
       <c r="C262" s="25"/>
       <c r="D262" s="25"/>
+      <c r="E262" s="15"/>
       <c r="F262" s="15">
         <v>1</v>
       </c>
@@ -12897,6 +13157,7 @@
       </c>
       <c r="C263" s="25"/>
       <c r="D263" s="25"/>
+      <c r="E263" s="15"/>
       <c r="F263" s="15">
         <v>1</v>
       </c>
@@ -12939,6 +13200,7 @@
       </c>
       <c r="C264" s="25"/>
       <c r="D264" s="25"/>
+      <c r="E264" s="15"/>
       <c r="F264" s="15">
         <v>1</v>
       </c>
@@ -12981,6 +13243,7 @@
       </c>
       <c r="C265" s="25"/>
       <c r="D265" s="25"/>
+      <c r="E265" s="15"/>
       <c r="F265" s="15">
         <v>1</v>
       </c>
@@ -13023,6 +13286,7 @@
       </c>
       <c r="C266" s="25"/>
       <c r="D266" s="25"/>
+      <c r="E266" s="15"/>
       <c r="F266" s="15">
         <v>1</v>
       </c>
@@ -13065,6 +13329,7 @@
       </c>
       <c r="C267" s="25"/>
       <c r="D267" s="25"/>
+      <c r="E267" s="15"/>
       <c r="F267" s="15">
         <v>1</v>
       </c>
@@ -13107,6 +13372,7 @@
       </c>
       <c r="C268" s="25"/>
       <c r="D268" s="25"/>
+      <c r="E268" s="15"/>
       <c r="F268" s="15">
         <v>1</v>
       </c>
@@ -13149,6 +13415,7 @@
       </c>
       <c r="C269" s="25"/>
       <c r="D269" s="25"/>
+      <c r="E269" s="15"/>
       <c r="F269" s="15">
         <v>1</v>
       </c>
@@ -13191,6 +13458,7 @@
       </c>
       <c r="C270" s="25"/>
       <c r="D270" s="25"/>
+      <c r="E270" s="15"/>
       <c r="F270" s="15">
         <v>1</v>
       </c>
@@ -13233,6 +13501,7 @@
       </c>
       <c r="C271" s="25"/>
       <c r="D271" s="25"/>
+      <c r="E271" s="15"/>
       <c r="F271" s="15">
         <v>1</v>
       </c>
@@ -13275,6 +13544,7 @@
       </c>
       <c r="C272" s="25"/>
       <c r="D272" s="25"/>
+      <c r="E272" s="15"/>
       <c r="F272" s="15">
         <v>1</v>
       </c>
@@ -13317,6 +13587,7 @@
       </c>
       <c r="C273" s="25"/>
       <c r="D273" s="25"/>
+      <c r="E273" s="15"/>
       <c r="F273" s="15">
         <v>1</v>
       </c>
@@ -13359,6 +13630,7 @@
       </c>
       <c r="C274" s="25"/>
       <c r="D274" s="25"/>
+      <c r="E274" s="15"/>
       <c r="F274" s="15">
         <v>1</v>
       </c>
@@ -13401,6 +13673,7 @@
       </c>
       <c r="C275" s="25"/>
       <c r="D275" s="25"/>
+      <c r="E275" s="15"/>
       <c r="F275" s="15">
         <v>1</v>
       </c>
@@ -13443,6 +13716,7 @@
       </c>
       <c r="C276" s="25"/>
       <c r="D276" s="25"/>
+      <c r="E276" s="15"/>
       <c r="F276" s="15">
         <v>1</v>
       </c>
@@ -13485,6 +13759,7 @@
       </c>
       <c r="C277" s="25"/>
       <c r="D277" s="25"/>
+      <c r="E277" s="15"/>
       <c r="F277" s="15">
         <v>1</v>
       </c>
@@ -13527,6 +13802,7 @@
       </c>
       <c r="C278" s="25"/>
       <c r="D278" s="25"/>
+      <c r="E278" s="15"/>
       <c r="F278" s="15">
         <v>1</v>
       </c>
@@ -13569,6 +13845,7 @@
       </c>
       <c r="C279" s="25"/>
       <c r="D279" s="25"/>
+      <c r="E279" s="15"/>
       <c r="F279" s="15">
         <v>1</v>
       </c>
@@ -13611,6 +13888,7 @@
       </c>
       <c r="C280" s="25"/>
       <c r="D280" s="25"/>
+      <c r="E280" s="15"/>
       <c r="F280" s="15">
         <v>1</v>
       </c>
@@ -13653,6 +13931,7 @@
       </c>
       <c r="C281" s="25"/>
       <c r="D281" s="25"/>
+      <c r="E281" s="15"/>
       <c r="F281" s="15">
         <v>1</v>
       </c>
@@ -13695,6 +13974,7 @@
       </c>
       <c r="C282" s="25"/>
       <c r="D282" s="25"/>
+      <c r="E282" s="15"/>
       <c r="F282" s="15">
         <v>1</v>
       </c>
@@ -13737,6 +14017,7 @@
       </c>
       <c r="C283" s="25"/>
       <c r="D283" s="25"/>
+      <c r="E283" s="15"/>
       <c r="F283" s="15">
         <v>1</v>
       </c>
@@ -13779,6 +14060,7 @@
       </c>
       <c r="C284" s="25"/>
       <c r="D284" s="25"/>
+      <c r="E284" s="15"/>
       <c r="F284" s="15">
         <v>1</v>
       </c>
@@ -13821,6 +14103,7 @@
       </c>
       <c r="C285" s="25"/>
       <c r="D285" s="25"/>
+      <c r="E285" s="15"/>
       <c r="F285" s="15">
         <v>1</v>
       </c>
@@ -13863,6 +14146,7 @@
       </c>
       <c r="C286" s="25"/>
       <c r="D286" s="25"/>
+      <c r="E286" s="15"/>
       <c r="F286" s="15">
         <v>1</v>
       </c>
@@ -13905,6 +14189,7 @@
       </c>
       <c r="C287" s="25"/>
       <c r="D287" s="25"/>
+      <c r="E287" s="15"/>
       <c r="F287" s="15">
         <v>1</v>
       </c>
@@ -13947,6 +14232,7 @@
       </c>
       <c r="C288" s="25"/>
       <c r="D288" s="25"/>
+      <c r="E288" s="15"/>
       <c r="F288" s="15">
         <v>1</v>
       </c>
@@ -13989,6 +14275,7 @@
       </c>
       <c r="C289" s="25"/>
       <c r="D289" s="25"/>
+      <c r="E289" s="15"/>
       <c r="F289" s="15">
         <v>1</v>
       </c>
@@ -14031,6 +14318,7 @@
       </c>
       <c r="C290" s="25"/>
       <c r="D290" s="25"/>
+      <c r="E290" s="15"/>
       <c r="F290" s="15">
         <v>1</v>
       </c>
@@ -14073,6 +14361,7 @@
       </c>
       <c r="C291" s="25"/>
       <c r="D291" s="25"/>
+      <c r="E291" s="15"/>
       <c r="F291" s="15">
         <v>1</v>
       </c>
@@ -14115,6 +14404,7 @@
       </c>
       <c r="C292" s="25"/>
       <c r="D292" s="25"/>
+      <c r="E292" s="15"/>
       <c r="F292" s="15">
         <v>1</v>
       </c>
@@ -14157,6 +14447,7 @@
       </c>
       <c r="C293" s="25"/>
       <c r="D293" s="25"/>
+      <c r="E293" s="15"/>
       <c r="F293" s="15">
         <v>1</v>
       </c>
@@ -14199,6 +14490,7 @@
       </c>
       <c r="C294" s="25"/>
       <c r="D294" s="25"/>
+      <c r="E294" s="15"/>
       <c r="F294" s="15">
         <v>1</v>
       </c>
@@ -14241,6 +14533,7 @@
       </c>
       <c r="C295" s="25"/>
       <c r="D295" s="25"/>
+      <c r="E295" s="15"/>
       <c r="F295" s="15">
         <v>1</v>
       </c>
@@ -14283,6 +14576,7 @@
       </c>
       <c r="C296" s="25"/>
       <c r="D296" s="25"/>
+      <c r="E296" s="15"/>
       <c r="F296" s="15">
         <v>1</v>
       </c>
@@ -14325,6 +14619,7 @@
       </c>
       <c r="C297" s="25"/>
       <c r="D297" s="25"/>
+      <c r="E297" s="15"/>
       <c r="F297" s="15">
         <v>1</v>
       </c>
@@ -14367,6 +14662,7 @@
       </c>
       <c r="C298" s="25"/>
       <c r="D298" s="25"/>
+      <c r="E298" s="15"/>
       <c r="F298" s="15">
         <v>1</v>
       </c>
@@ -14409,6 +14705,7 @@
       </c>
       <c r="C299" s="25"/>
       <c r="D299" s="25"/>
+      <c r="E299" s="15"/>
       <c r="F299" s="15">
         <v>1</v>
       </c>
@@ -14451,6 +14748,7 @@
       </c>
       <c r="C300" s="25"/>
       <c r="D300" s="25"/>
+      <c r="E300" s="15"/>
       <c r="F300" s="15">
         <v>1</v>
       </c>
@@ -14493,6 +14791,7 @@
       </c>
       <c r="C301" s="25"/>
       <c r="D301" s="25"/>
+      <c r="E301" s="15"/>
       <c r="F301" s="15">
         <v>1</v>
       </c>
@@ -14535,6 +14834,7 @@
       </c>
       <c r="C302" s="25"/>
       <c r="D302" s="25"/>
+      <c r="E302" s="15"/>
       <c r="F302" s="15">
         <v>1</v>
       </c>
@@ -14577,6 +14877,7 @@
       </c>
       <c r="C303" s="25"/>
       <c r="D303" s="25"/>
+      <c r="E303" s="15"/>
       <c r="F303" s="15">
         <v>1</v>
       </c>
@@ -14619,6 +14920,7 @@
       </c>
       <c r="C304" s="25"/>
       <c r="D304" s="25"/>
+      <c r="E304" s="15"/>
       <c r="F304" s="15">
         <v>1</v>
       </c>
@@ -14661,6 +14963,7 @@
       </c>
       <c r="C305" s="25"/>
       <c r="D305" s="25"/>
+      <c r="E305" s="15"/>
       <c r="F305" s="15">
         <v>1</v>
       </c>
@@ -14703,6 +15006,7 @@
       </c>
       <c r="C306" s="25"/>
       <c r="D306" s="25"/>
+      <c r="E306" s="15"/>
       <c r="F306" s="15">
         <v>1</v>
       </c>
@@ -14745,6 +15049,7 @@
       </c>
       <c r="C307" s="25"/>
       <c r="D307" s="25"/>
+      <c r="E307" s="15"/>
       <c r="F307" s="15">
         <v>1</v>
       </c>
@@ -14787,6 +15092,7 @@
       </c>
       <c r="C308" s="25"/>
       <c r="D308" s="25"/>
+      <c r="E308" s="15"/>
       <c r="F308" s="15">
         <v>1</v>
       </c>
@@ -14829,6 +15135,7 @@
       </c>
       <c r="C309" s="25"/>
       <c r="D309" s="25"/>
+      <c r="E309" s="15"/>
       <c r="F309" s="15">
         <v>1</v>
       </c>
@@ -14871,6 +15178,7 @@
       </c>
       <c r="C310" s="25"/>
       <c r="D310" s="25"/>
+      <c r="E310" s="15"/>
       <c r="F310" s="15">
         <v>1</v>
       </c>
@@ -14913,6 +15221,7 @@
       </c>
       <c r="C311" s="25"/>
       <c r="D311" s="25"/>
+      <c r="E311" s="15"/>
       <c r="F311" s="15">
         <v>1</v>
       </c>
@@ -14955,6 +15264,7 @@
       </c>
       <c r="C312" s="25"/>
       <c r="D312" s="25"/>
+      <c r="E312" s="15"/>
       <c r="F312" s="15">
         <v>1</v>
       </c>
@@ -14997,6 +15307,7 @@
       </c>
       <c r="C313" s="25"/>
       <c r="D313" s="25"/>
+      <c r="E313" s="15"/>
       <c r="F313" s="15">
         <v>1</v>
       </c>
@@ -15039,6 +15350,7 @@
       </c>
       <c r="C314" s="25"/>
       <c r="D314" s="25"/>
+      <c r="E314" s="15"/>
       <c r="F314" s="15">
         <v>1</v>
       </c>
@@ -15081,6 +15393,7 @@
       </c>
       <c r="C315" s="25"/>
       <c r="D315" s="25"/>
+      <c r="E315" s="15"/>
       <c r="F315" s="15">
         <v>1</v>
       </c>
@@ -15123,6 +15436,7 @@
       </c>
       <c r="C316" s="25"/>
       <c r="D316" s="25"/>
+      <c r="E316" s="15"/>
       <c r="F316" s="15">
         <v>1</v>
       </c>
@@ -15165,6 +15479,7 @@
       </c>
       <c r="C317" s="25"/>
       <c r="D317" s="25"/>
+      <c r="E317" s="15"/>
       <c r="F317" s="15">
         <v>1</v>
       </c>
@@ -15207,6 +15522,7 @@
       </c>
       <c r="C318" s="25"/>
       <c r="D318" s="25"/>
+      <c r="E318" s="15"/>
       <c r="F318" s="15">
         <v>1</v>
       </c>
@@ -15249,6 +15565,7 @@
       </c>
       <c r="C319" s="25"/>
       <c r="D319" s="25"/>
+      <c r="E319" s="15"/>
       <c r="F319" s="15">
         <v>1</v>
       </c>
@@ -15291,6 +15608,7 @@
       </c>
       <c r="C320" s="25"/>
       <c r="D320" s="25"/>
+      <c r="E320" s="15"/>
       <c r="F320" s="15">
         <v>1</v>
       </c>
@@ -15333,6 +15651,7 @@
       </c>
       <c r="C321" s="25"/>
       <c r="D321" s="25"/>
+      <c r="E321" s="15"/>
       <c r="F321" s="15">
         <v>1</v>
       </c>
@@ -15375,6 +15694,7 @@
       </c>
       <c r="C322" s="25"/>
       <c r="D322" s="25"/>
+      <c r="E322" s="15"/>
       <c r="F322" s="15">
         <v>1</v>
       </c>
@@ -15417,6 +15737,7 @@
       </c>
       <c r="C323" s="25"/>
       <c r="D323" s="25"/>
+      <c r="E323" s="15"/>
       <c r="F323" s="15">
         <v>1</v>
       </c>
@@ -15459,6 +15780,7 @@
       </c>
       <c r="C324" s="25"/>
       <c r="D324" s="25"/>
+      <c r="E324" s="15"/>
       <c r="F324" s="15">
         <v>1</v>
       </c>
@@ -15501,6 +15823,7 @@
       </c>
       <c r="C325" s="25"/>
       <c r="D325" s="25"/>
+      <c r="E325" s="15"/>
       <c r="F325" s="15">
         <v>1</v>
       </c>
@@ -15543,6 +15866,7 @@
       </c>
       <c r="C326" s="25"/>
       <c r="D326" s="25"/>
+      <c r="E326" s="15"/>
       <c r="F326" s="15">
         <v>1</v>
       </c>
@@ -15585,6 +15909,7 @@
       </c>
       <c r="C327" s="25"/>
       <c r="D327" s="25"/>
+      <c r="E327" s="15"/>
       <c r="F327" s="15">
         <v>1</v>
       </c>
@@ -15627,6 +15952,7 @@
       </c>
       <c r="C328" s="25"/>
       <c r="D328" s="25"/>
+      <c r="E328" s="15"/>
       <c r="F328" s="15">
         <v>1</v>
       </c>
@@ -15669,6 +15995,7 @@
       </c>
       <c r="C329" s="25"/>
       <c r="D329" s="25"/>
+      <c r="E329" s="15"/>
       <c r="F329" s="15">
         <v>1</v>
       </c>
@@ -15711,6 +16038,7 @@
       </c>
       <c r="C330" s="25"/>
       <c r="D330" s="25"/>
+      <c r="E330" s="15"/>
       <c r="F330" s="15">
         <v>1</v>
       </c>
@@ -15753,6 +16081,7 @@
       </c>
       <c r="C331" s="25"/>
       <c r="D331" s="25"/>
+      <c r="E331" s="15"/>
       <c r="F331" s="15">
         <v>1</v>
       </c>
@@ -15795,6 +16124,7 @@
       </c>
       <c r="C332" s="25"/>
       <c r="D332" s="25"/>
+      <c r="E332" s="15"/>
       <c r="F332" s="15">
         <v>1</v>
       </c>
@@ -15837,6 +16167,7 @@
       </c>
       <c r="C333" s="25"/>
       <c r="D333" s="25"/>
+      <c r="E333" s="15"/>
       <c r="F333" s="15">
         <v>1</v>
       </c>
@@ -15879,6 +16210,7 @@
       </c>
       <c r="C334" s="25"/>
       <c r="D334" s="25"/>
+      <c r="E334" s="15"/>
       <c r="F334" s="15">
         <v>1</v>
       </c>
@@ -15921,6 +16253,7 @@
       </c>
       <c r="C335" s="25"/>
       <c r="D335" s="25"/>
+      <c r="E335" s="15"/>
       <c r="F335" s="15">
         <v>1</v>
       </c>
@@ -15963,6 +16296,7 @@
       </c>
       <c r="C336" s="25"/>
       <c r="D336" s="25"/>
+      <c r="E336" s="15"/>
       <c r="F336" s="15">
         <v>1</v>
       </c>
@@ -16005,6 +16339,7 @@
       </c>
       <c r="C337" s="25"/>
       <c r="D337" s="25"/>
+      <c r="E337" s="15"/>
       <c r="F337" s="15">
         <v>1</v>
       </c>
@@ -16047,6 +16382,7 @@
       </c>
       <c r="C338" s="25"/>
       <c r="D338" s="25"/>
+      <c r="E338" s="15"/>
       <c r="F338" s="15">
         <v>1</v>
       </c>
@@ -16089,6 +16425,7 @@
       </c>
       <c r="C339" s="25"/>
       <c r="D339" s="25"/>
+      <c r="E339" s="15"/>
       <c r="F339" s="15">
         <v>1</v>
       </c>
@@ -16131,6 +16468,7 @@
       </c>
       <c r="C340" s="25"/>
       <c r="D340" s="25"/>
+      <c r="E340" s="15"/>
       <c r="F340" s="15">
         <v>1</v>
       </c>
@@ -16173,6 +16511,7 @@
       </c>
       <c r="C341" s="25"/>
       <c r="D341" s="25"/>
+      <c r="E341" s="15"/>
       <c r="F341" s="15">
         <v>1</v>
       </c>
@@ -16215,6 +16554,7 @@
       </c>
       <c r="C342" s="25"/>
       <c r="D342" s="25"/>
+      <c r="E342" s="15"/>
       <c r="F342" s="15">
         <v>1</v>
       </c>
@@ -16257,6 +16597,7 @@
       </c>
       <c r="C343" s="25"/>
       <c r="D343" s="25"/>
+      <c r="E343" s="15"/>
       <c r="F343" s="15">
         <v>1</v>
       </c>
@@ -16299,6 +16640,7 @@
       </c>
       <c r="C344" s="25"/>
       <c r="D344" s="25"/>
+      <c r="E344" s="15"/>
       <c r="F344" s="15">
         <v>1</v>
       </c>
@@ -16341,6 +16683,7 @@
       </c>
       <c r="C345" s="25"/>
       <c r="D345" s="25"/>
+      <c r="E345" s="15"/>
       <c r="F345" s="15">
         <v>1</v>
       </c>
@@ -16383,6 +16726,7 @@
       </c>
       <c r="C346" s="25"/>
       <c r="D346" s="25"/>
+      <c r="E346" s="15"/>
       <c r="F346" s="15">
         <v>1</v>
       </c>
@@ -16425,6 +16769,7 @@
       </c>
       <c r="C347" s="25"/>
       <c r="D347" s="25"/>
+      <c r="E347" s="15"/>
       <c r="F347" s="15">
         <v>1</v>
       </c>
@@ -16467,6 +16812,7 @@
       </c>
       <c r="C348" s="25"/>
       <c r="D348" s="25"/>
+      <c r="E348" s="15"/>
       <c r="F348" s="15">
         <v>1</v>
       </c>
@@ -16509,6 +16855,7 @@
       </c>
       <c r="C349" s="25"/>
       <c r="D349" s="25"/>
+      <c r="E349" s="15"/>
       <c r="F349" s="15">
         <v>1</v>
       </c>
@@ -16551,6 +16898,7 @@
       </c>
       <c r="C350" s="25"/>
       <c r="D350" s="25"/>
+      <c r="E350" s="15"/>
       <c r="F350" s="15">
         <v>1</v>
       </c>
@@ -16593,6 +16941,7 @@
       </c>
       <c r="C351" s="25"/>
       <c r="D351" s="25"/>
+      <c r="E351" s="15"/>
       <c r="F351" s="15">
         <v>1</v>
       </c>
@@ -16635,6 +16984,7 @@
       </c>
       <c r="C352" s="25"/>
       <c r="D352" s="25"/>
+      <c r="E352" s="15"/>
       <c r="F352" s="15">
         <v>1</v>
       </c>
@@ -16677,6 +17027,7 @@
       </c>
       <c r="C353" s="25"/>
       <c r="D353" s="25"/>
+      <c r="E353" s="15"/>
       <c r="F353" s="15">
         <v>1</v>
       </c>
@@ -16719,6 +17070,7 @@
       </c>
       <c r="C354" s="25"/>
       <c r="D354" s="25"/>
+      <c r="E354" s="15"/>
       <c r="F354" s="15">
         <v>1</v>
       </c>
@@ -16761,6 +17113,7 @@
       </c>
       <c r="C355" s="25"/>
       <c r="D355" s="25"/>
+      <c r="E355" s="15"/>
       <c r="F355" s="15">
         <v>1</v>
       </c>
@@ -16803,6 +17156,7 @@
       </c>
       <c r="C356" s="25"/>
       <c r="D356" s="25"/>
+      <c r="E356" s="15"/>
       <c r="F356" s="15">
         <v>1</v>
       </c>
@@ -16845,6 +17199,7 @@
       </c>
       <c r="C357" s="25"/>
       <c r="D357" s="25"/>
+      <c r="E357" s="15"/>
       <c r="F357" s="15">
         <v>1</v>
       </c>
@@ -16887,6 +17242,7 @@
       </c>
       <c r="C358" s="25"/>
       <c r="D358" s="25"/>
+      <c r="E358" s="15"/>
       <c r="F358" s="15">
         <v>1</v>
       </c>
@@ -16929,6 +17285,7 @@
       </c>
       <c r="C359" s="25"/>
       <c r="D359" s="25"/>
+      <c r="E359" s="15"/>
       <c r="F359" s="15">
         <v>1</v>
       </c>
@@ -16971,6 +17328,7 @@
       </c>
       <c r="C360" s="25"/>
       <c r="D360" s="25"/>
+      <c r="E360" s="15"/>
       <c r="F360" s="15">
         <v>1</v>
       </c>
@@ -17013,6 +17371,7 @@
       </c>
       <c r="C361" s="25"/>
       <c r="D361" s="25"/>
+      <c r="E361" s="15"/>
       <c r="F361" s="15">
         <v>1</v>
       </c>
@@ -17055,6 +17414,7 @@
       </c>
       <c r="C362" s="25"/>
       <c r="D362" s="25"/>
+      <c r="E362" s="15"/>
       <c r="F362" s="15">
         <v>1</v>
       </c>
@@ -17097,6 +17457,7 @@
       </c>
       <c r="C363" s="25"/>
       <c r="D363" s="25"/>
+      <c r="E363" s="15"/>
       <c r="F363" s="15">
         <v>1</v>
       </c>
@@ -17139,6 +17500,7 @@
       </c>
       <c r="C364" s="25"/>
       <c r="D364" s="25"/>
+      <c r="E364" s="15"/>
       <c r="F364" s="15">
         <v>1</v>
       </c>
@@ -17181,6 +17543,7 @@
       </c>
       <c r="C365" s="25"/>
       <c r="D365" s="25"/>
+      <c r="E365" s="15"/>
       <c r="F365" s="15">
         <v>1</v>
       </c>
@@ -17223,6 +17586,7 @@
       </c>
       <c r="C366" s="25"/>
       <c r="D366" s="25"/>
+      <c r="E366" s="15"/>
       <c r="F366" s="15">
         <v>1</v>
       </c>
@@ -17265,6 +17629,7 @@
       </c>
       <c r="C367" s="25"/>
       <c r="D367" s="25"/>
+      <c r="E367" s="15"/>
       <c r="F367" s="15">
         <v>1</v>
       </c>
@@ -17307,6 +17672,7 @@
       </c>
       <c r="C368" s="25"/>
       <c r="D368" s="25"/>
+      <c r="E368" s="15"/>
       <c r="F368" s="15">
         <v>1</v>
       </c>
@@ -17349,6 +17715,7 @@
       </c>
       <c r="C369" s="25"/>
       <c r="D369" s="25"/>
+      <c r="E369" s="15"/>
       <c r="F369" s="15">
         <v>1</v>
       </c>
@@ -17391,6 +17758,7 @@
       </c>
       <c r="C370" s="25"/>
       <c r="D370" s="25"/>
+      <c r="E370" s="15"/>
       <c r="F370" s="15">
         <v>1</v>
       </c>
@@ -17433,6 +17801,7 @@
       </c>
       <c r="C371" s="25"/>
       <c r="D371" s="25"/>
+      <c r="E371" s="15"/>
       <c r="F371" s="15">
         <v>1</v>
       </c>
@@ -17475,6 +17844,7 @@
       </c>
       <c r="C372" s="25"/>
       <c r="D372" s="25"/>
+      <c r="E372" s="15"/>
       <c r="F372" s="15">
         <v>1</v>
       </c>
@@ -17517,6 +17887,7 @@
       </c>
       <c r="C373" s="25"/>
       <c r="D373" s="25"/>
+      <c r="E373" s="15"/>
       <c r="F373" s="15">
         <v>1</v>
       </c>
@@ -17559,6 +17930,7 @@
       </c>
       <c r="C374" s="25"/>
       <c r="D374" s="25"/>
+      <c r="E374" s="15"/>
       <c r="F374" s="15">
         <v>1</v>
       </c>
@@ -17601,6 +17973,7 @@
       </c>
       <c r="C375" s="25"/>
       <c r="D375" s="25"/>
+      <c r="E375" s="15"/>
       <c r="F375" s="15">
         <v>1</v>
       </c>
@@ -17643,6 +18016,7 @@
       </c>
       <c r="C376" s="25"/>
       <c r="D376" s="25"/>
+      <c r="E376" s="15"/>
       <c r="F376" s="15">
         <v>1</v>
       </c>
@@ -17685,6 +18059,7 @@
       </c>
       <c r="C377" s="25"/>
       <c r="D377" s="25"/>
+      <c r="E377" s="15"/>
       <c r="F377" s="15">
         <v>1</v>
       </c>
@@ -17727,6 +18102,7 @@
       </c>
       <c r="C378" s="25"/>
       <c r="D378" s="25"/>
+      <c r="E378" s="15"/>
       <c r="F378" s="15">
         <v>1</v>
       </c>
@@ -17769,6 +18145,7 @@
       </c>
       <c r="C379" s="25"/>
       <c r="D379" s="25"/>
+      <c r="E379" s="15"/>
       <c r="F379" s="15">
         <v>1</v>
       </c>
@@ -17811,6 +18188,7 @@
       </c>
       <c r="C380" s="25"/>
       <c r="D380" s="25"/>
+      <c r="E380" s="15"/>
       <c r="F380" s="15">
         <v>1</v>
       </c>
@@ -17853,6 +18231,7 @@
       </c>
       <c r="C381" s="25"/>
       <c r="D381" s="25"/>
+      <c r="E381" s="15"/>
       <c r="F381" s="15">
         <v>1</v>
       </c>
@@ -17895,6 +18274,7 @@
       </c>
       <c r="C382" s="25"/>
       <c r="D382" s="25"/>
+      <c r="E382" s="15"/>
       <c r="F382" s="15">
         <v>1</v>
       </c>
@@ -17937,6 +18317,7 @@
       </c>
       <c r="C383" s="25"/>
       <c r="D383" s="25"/>
+      <c r="E383" s="15"/>
       <c r="F383" s="15">
         <v>1</v>
       </c>
@@ -17979,6 +18360,7 @@
       </c>
       <c r="C384" s="25"/>
       <c r="D384" s="25"/>
+      <c r="E384" s="15"/>
       <c r="F384" s="15">
         <v>1</v>
       </c>
@@ -18021,6 +18403,7 @@
       </c>
       <c r="C385" s="25"/>
       <c r="D385" s="25"/>
+      <c r="E385" s="15"/>
       <c r="F385" s="15">
         <v>1</v>
       </c>
@@ -18063,6 +18446,7 @@
       </c>
       <c r="C386" s="25"/>
       <c r="D386" s="25"/>
+      <c r="E386" s="15"/>
       <c r="F386" s="15">
         <v>1</v>
       </c>
@@ -18105,6 +18489,7 @@
       </c>
       <c r="C387" s="25"/>
       <c r="D387" s="25"/>
+      <c r="E387" s="15"/>
       <c r="F387" s="15">
         <v>1</v>
       </c>
@@ -18147,6 +18532,7 @@
       </c>
       <c r="C388" s="25"/>
       <c r="D388" s="25"/>
+      <c r="E388" s="15"/>
       <c r="F388" s="15">
         <v>1</v>
       </c>
@@ -18189,6 +18575,7 @@
       </c>
       <c r="C389" s="25"/>
       <c r="D389" s="25"/>
+      <c r="E389" s="15"/>
       <c r="F389" s="15">
         <v>1</v>
       </c>
@@ -18231,6 +18618,7 @@
       </c>
       <c r="C390" s="25"/>
       <c r="D390" s="25"/>
+      <c r="E390" s="15"/>
       <c r="F390" s="15">
         <v>1</v>
       </c>
@@ -18273,6 +18661,7 @@
       </c>
       <c r="C391" s="25"/>
       <c r="D391" s="25"/>
+      <c r="E391" s="15"/>
       <c r="F391" s="15">
         <v>1</v>
       </c>
@@ -18315,6 +18704,7 @@
       </c>
       <c r="C392" s="25"/>
       <c r="D392" s="25"/>
+      <c r="E392" s="15"/>
       <c r="F392" s="15">
         <v>1</v>
       </c>
@@ -18357,6 +18747,7 @@
       </c>
       <c r="C393" s="25"/>
       <c r="D393" s="25"/>
+      <c r="E393" s="15"/>
       <c r="F393" s="15">
         <v>1</v>
       </c>
@@ -18399,6 +18790,7 @@
       </c>
       <c r="C394" s="25"/>
       <c r="D394" s="25"/>
+      <c r="E394" s="15"/>
       <c r="F394" s="15">
         <v>1</v>
       </c>
@@ -18441,6 +18833,7 @@
       </c>
       <c r="C395" s="25"/>
       <c r="D395" s="25"/>
+      <c r="E395" s="15"/>
       <c r="F395" s="15">
         <v>1</v>
       </c>
@@ -18483,6 +18876,7 @@
       </c>
       <c r="C396" s="25"/>
       <c r="D396" s="25"/>
+      <c r="E396" s="15"/>
       <c r="F396" s="15">
         <v>1</v>
       </c>
@@ -18525,6 +18919,7 @@
       </c>
       <c r="C397" s="25"/>
       <c r="D397" s="25"/>
+      <c r="E397" s="15"/>
       <c r="F397" s="15">
         <v>1</v>
       </c>
@@ -18567,6 +18962,7 @@
       </c>
       <c r="C398" s="25"/>
       <c r="D398" s="25"/>
+      <c r="E398" s="15"/>
       <c r="F398" s="15">
         <v>1</v>
       </c>
@@ -18609,6 +19005,7 @@
       </c>
       <c r="C399" s="25"/>
       <c r="D399" s="25"/>
+      <c r="E399" s="15"/>
       <c r="F399" s="15">
         <v>1</v>
       </c>
@@ -18651,6 +19048,7 @@
       </c>
       <c r="C400" s="25"/>
       <c r="D400" s="25"/>
+      <c r="E400" s="15"/>
       <c r="F400" s="15">
         <v>1</v>
       </c>
@@ -18693,6 +19091,7 @@
       </c>
       <c r="C401" s="25"/>
       <c r="D401" s="25"/>
+      <c r="E401" s="15"/>
       <c r="F401" s="15">
         <v>1</v>
       </c>
@@ -18735,6 +19134,7 @@
       </c>
       <c r="C402" s="25"/>
       <c r="D402" s="25"/>
+      <c r="E402" s="15"/>
       <c r="F402" s="15">
         <v>1</v>
       </c>
@@ -18777,6 +19177,7 @@
       </c>
       <c r="C403" s="25"/>
       <c r="D403" s="25"/>
+      <c r="E403" s="15"/>
       <c r="F403" s="15">
         <v>1</v>
       </c>
@@ -18819,6 +19220,7 @@
       </c>
       <c r="C404" s="25"/>
       <c r="D404" s="25"/>
+      <c r="E404" s="15"/>
       <c r="F404" s="15">
         <v>1</v>
       </c>
@@ -18861,6 +19263,7 @@
       </c>
       <c r="C405" s="25"/>
       <c r="D405" s="25"/>
+      <c r="E405" s="15"/>
       <c r="F405" s="15">
         <v>1</v>
       </c>
@@ -18903,6 +19306,7 @@
       </c>
       <c r="C406" s="25"/>
       <c r="D406" s="25"/>
+      <c r="E406" s="15"/>
       <c r="F406" s="15">
         <v>1</v>
       </c>
@@ -18945,6 +19349,7 @@
       </c>
       <c r="C407" s="25"/>
       <c r="D407" s="25"/>
+      <c r="E407" s="15"/>
       <c r="F407" s="15">
         <v>1</v>
       </c>
@@ -18987,6 +19392,7 @@
       </c>
       <c r="C408" s="25"/>
       <c r="D408" s="25"/>
+      <c r="E408" s="15"/>
       <c r="F408" s="15">
         <v>1</v>
       </c>
@@ -19029,6 +19435,7 @@
       </c>
       <c r="C409" s="25"/>
       <c r="D409" s="25"/>
+      <c r="E409" s="15"/>
       <c r="F409" s="15">
         <v>1</v>
       </c>
@@ -19071,6 +19478,7 @@
       </c>
       <c r="C410" s="25"/>
       <c r="D410" s="25"/>
+      <c r="E410" s="15"/>
       <c r="F410" s="15">
         <v>1</v>
       </c>
@@ -19113,6 +19521,7 @@
       </c>
       <c r="C411" s="25"/>
       <c r="D411" s="25"/>
+      <c r="E411" s="15"/>
       <c r="F411" s="15">
         <v>1</v>
       </c>
@@ -19155,6 +19564,7 @@
       </c>
       <c r="C412" s="25"/>
       <c r="D412" s="25"/>
+      <c r="E412" s="15"/>
       <c r="F412" s="15">
         <v>1</v>
       </c>
@@ -19197,6 +19607,7 @@
       </c>
       <c r="C413" s="25"/>
       <c r="D413" s="25"/>
+      <c r="E413" s="15"/>
       <c r="F413" s="15">
         <v>1</v>
       </c>
@@ -19239,6 +19650,7 @@
       </c>
       <c r="C414" s="25"/>
       <c r="D414" s="25"/>
+      <c r="E414" s="15"/>
       <c r="F414" s="15">
         <v>1</v>
       </c>
@@ -19281,6 +19693,7 @@
       </c>
       <c r="C415" s="25"/>
       <c r="D415" s="25"/>
+      <c r="E415" s="15"/>
       <c r="F415" s="15">
         <v>1</v>
       </c>
@@ -19323,6 +19736,7 @@
       </c>
       <c r="C416" s="25"/>
       <c r="D416" s="25"/>
+      <c r="E416" s="15"/>
       <c r="F416" s="15">
         <v>1</v>
       </c>
@@ -19365,6 +19779,7 @@
       </c>
       <c r="C417" s="25"/>
       <c r="D417" s="25"/>
+      <c r="E417" s="15"/>
       <c r="F417" s="15">
         <v>1</v>
       </c>
@@ -19407,6 +19822,7 @@
       </c>
       <c r="C418" s="25"/>
       <c r="D418" s="25"/>
+      <c r="E418" s="15"/>
       <c r="F418" s="15">
         <v>1</v>
       </c>
@@ -19449,6 +19865,7 @@
       </c>
       <c r="C419" s="25"/>
       <c r="D419" s="25"/>
+      <c r="E419" s="15"/>
       <c r="F419" s="15">
         <v>1</v>
       </c>
@@ -19491,6 +19908,7 @@
       </c>
       <c r="C420" s="25"/>
       <c r="D420" s="25"/>
+      <c r="E420" s="15"/>
       <c r="F420" s="15">
         <v>1</v>
       </c>
@@ -19533,6 +19951,7 @@
       </c>
       <c r="C421" s="25"/>
       <c r="D421" s="25"/>
+      <c r="E421" s="15"/>
       <c r="F421" s="15">
         <v>1</v>
       </c>
@@ -19575,6 +19994,7 @@
       </c>
       <c r="C422" s="25"/>
       <c r="D422" s="25"/>
+      <c r="E422" s="15"/>
       <c r="F422" s="15">
         <v>1</v>
       </c>
@@ -19617,6 +20037,7 @@
       </c>
       <c r="C423" s="25"/>
       <c r="D423" s="25"/>
+      <c r="E423" s="15"/>
       <c r="F423" s="15">
         <v>1</v>
       </c>
@@ -19659,6 +20080,7 @@
       </c>
       <c r="C424" s="25"/>
       <c r="D424" s="25"/>
+      <c r="E424" s="15"/>
       <c r="F424" s="15">
         <v>1</v>
       </c>
@@ -19701,6 +20123,7 @@
       </c>
       <c r="C425" s="25"/>
       <c r="D425" s="25"/>
+      <c r="E425" s="15"/>
       <c r="F425" s="15">
         <v>1</v>
       </c>
@@ -19743,6 +20166,7 @@
       </c>
       <c r="C426" s="25"/>
       <c r="D426" s="25"/>
+      <c r="E426" s="15"/>
       <c r="F426" s="15">
         <v>1</v>
       </c>
@@ -19785,6 +20209,7 @@
       </c>
       <c r="C427" s="25"/>
       <c r="D427" s="25"/>
+      <c r="E427" s="15"/>
       <c r="F427" s="15">
         <v>1</v>
       </c>
@@ -19827,6 +20252,7 @@
       </c>
       <c r="C428" s="25"/>
       <c r="D428" s="25"/>
+      <c r="E428" s="15"/>
       <c r="F428" s="15">
         <v>1</v>
       </c>
@@ -19869,6 +20295,7 @@
       </c>
       <c r="C429" s="25"/>
       <c r="D429" s="25"/>
+      <c r="E429" s="15"/>
       <c r="F429" s="15">
         <v>1</v>
       </c>
@@ -19911,6 +20338,7 @@
       </c>
       <c r="C430" s="25"/>
       <c r="D430" s="25"/>
+      <c r="E430" s="15"/>
       <c r="F430" s="15">
         <v>1</v>
       </c>
@@ -19953,6 +20381,7 @@
       </c>
       <c r="C431" s="25"/>
       <c r="D431" s="25"/>
+      <c r="E431" s="15"/>
       <c r="F431" s="15">
         <v>1</v>
       </c>
@@ -19995,6 +20424,7 @@
       </c>
       <c r="C432" s="25"/>
       <c r="D432" s="25"/>
+      <c r="E432" s="15"/>
       <c r="F432" s="15">
         <v>1</v>
       </c>
@@ -20037,6 +20467,7 @@
       </c>
       <c r="C433" s="25"/>
       <c r="D433" s="25"/>
+      <c r="E433" s="15"/>
       <c r="F433" s="15">
         <v>1</v>
       </c>
@@ -20079,6 +20510,7 @@
       </c>
       <c r="C434" s="25"/>
       <c r="D434" s="25"/>
+      <c r="E434" s="15"/>
       <c r="F434" s="15">
         <v>1</v>
       </c>
@@ -20121,6 +20553,7 @@
       </c>
       <c r="C435" s="25"/>
       <c r="D435" s="25"/>
+      <c r="E435" s="15"/>
       <c r="F435" s="15">
         <v>1</v>
       </c>
@@ -20163,6 +20596,7 @@
       </c>
       <c r="C436" s="25"/>
       <c r="D436" s="25"/>
+      <c r="E436" s="15"/>
       <c r="F436" s="15">
         <v>1</v>
       </c>
@@ -20205,6 +20639,7 @@
       </c>
       <c r="C437" s="25"/>
       <c r="D437" s="25"/>
+      <c r="E437" s="15"/>
       <c r="F437" s="15">
         <v>1</v>
       </c>
@@ -20247,6 +20682,7 @@
       </c>
       <c r="C438" s="25"/>
       <c r="D438" s="25"/>
+      <c r="E438" s="15"/>
       <c r="F438" s="15">
         <v>1</v>
       </c>
@@ -20289,6 +20725,7 @@
       </c>
       <c r="C439" s="25"/>
       <c r="D439" s="25"/>
+      <c r="E439" s="15"/>
       <c r="F439" s="15">
         <v>1</v>
       </c>
@@ -20331,6 +20768,7 @@
       </c>
       <c r="C440" s="25"/>
       <c r="D440" s="25"/>
+      <c r="E440" s="15"/>
       <c r="F440" s="15">
         <v>1</v>
       </c>
@@ -20373,6 +20811,7 @@
       </c>
       <c r="C441" s="25"/>
       <c r="D441" s="25"/>
+      <c r="E441" s="15"/>
       <c r="F441" s="15">
         <v>1</v>
       </c>
@@ -20415,6 +20854,7 @@
       </c>
       <c r="C442" s="25"/>
       <c r="D442" s="25"/>
+      <c r="E442" s="15"/>
       <c r="F442" s="15">
         <v>1</v>
       </c>
@@ -20457,6 +20897,7 @@
       </c>
       <c r="C443" s="25"/>
       <c r="D443" s="25"/>
+      <c r="E443" s="15"/>
       <c r="F443" s="15">
         <v>1</v>
       </c>
@@ -20499,6 +20940,7 @@
       </c>
       <c r="C444" s="25"/>
       <c r="D444" s="25"/>
+      <c r="E444" s="15"/>
       <c r="F444" s="15">
         <v>1</v>
       </c>
@@ -20541,6 +20983,7 @@
       </c>
       <c r="C445" s="25"/>
       <c r="D445" s="25"/>
+      <c r="E445" s="15"/>
       <c r="F445" s="15">
         <v>1</v>
       </c>
@@ -20583,6 +21026,7 @@
       </c>
       <c r="C446" s="25"/>
       <c r="D446" s="25"/>
+      <c r="E446" s="15"/>
       <c r="F446" s="15">
         <v>1</v>
       </c>
@@ -20625,6 +21069,7 @@
       </c>
       <c r="C447" s="25"/>
       <c r="D447" s="25"/>
+      <c r="E447" s="15"/>
       <c r="F447" s="15">
         <v>1</v>
       </c>
@@ -20667,6 +21112,7 @@
       </c>
       <c r="C448" s="25"/>
       <c r="D448" s="25"/>
+      <c r="E448" s="15"/>
       <c r="F448" s="15">
         <v>1</v>
       </c>
@@ -20709,6 +21155,7 @@
       </c>
       <c r="C449" s="25"/>
       <c r="D449" s="25"/>
+      <c r="E449" s="15"/>
       <c r="F449" s="15">
         <v>1</v>
       </c>
@@ -20751,6 +21198,7 @@
       </c>
       <c r="C450" s="25"/>
       <c r="D450" s="25"/>
+      <c r="E450" s="15"/>
       <c r="F450" s="15">
         <v>1</v>
       </c>
@@ -20793,6 +21241,7 @@
       </c>
       <c r="C451" s="25"/>
       <c r="D451" s="25"/>
+      <c r="E451" s="15"/>
       <c r="F451" s="15">
         <v>1</v>
       </c>
@@ -20835,6 +21284,7 @@
       </c>
       <c r="C452" s="25"/>
       <c r="D452" s="25"/>
+      <c r="E452" s="15"/>
       <c r="F452" s="15">
         <v>1</v>
       </c>
@@ -20877,6 +21327,7 @@
       </c>
       <c r="C453" s="25"/>
       <c r="D453" s="25"/>
+      <c r="E453" s="15"/>
       <c r="F453" s="15">
         <v>1</v>
       </c>
@@ -20919,6 +21370,7 @@
       </c>
       <c r="C454" s="25"/>
       <c r="D454" s="25"/>
+      <c r="E454" s="15"/>
       <c r="F454" s="15">
         <v>1</v>
       </c>
@@ -20961,6 +21413,7 @@
       </c>
       <c r="C455" s="25"/>
       <c r="D455" s="25"/>
+      <c r="E455" s="15"/>
       <c r="F455" s="15">
         <v>1</v>
       </c>
@@ -21003,6 +21456,7 @@
       </c>
       <c r="C456" s="25"/>
       <c r="D456" s="25"/>
+      <c r="E456" s="15"/>
       <c r="F456" s="15">
         <v>1</v>
       </c>
@@ -21045,6 +21499,7 @@
       </c>
       <c r="C457" s="25"/>
       <c r="D457" s="25"/>
+      <c r="E457" s="15"/>
       <c r="F457" s="15">
         <v>1</v>
       </c>
@@ -21087,6 +21542,7 @@
       </c>
       <c r="C458" s="25"/>
       <c r="D458" s="25"/>
+      <c r="E458" s="15"/>
       <c r="F458" s="15">
         <v>1</v>
       </c>
@@ -21129,6 +21585,7 @@
       </c>
       <c r="C459" s="25"/>
       <c r="D459" s="25"/>
+      <c r="E459" s="15"/>
       <c r="F459" s="15">
         <v>1</v>
       </c>
@@ -21171,6 +21628,7 @@
       </c>
       <c r="C460" s="25"/>
       <c r="D460" s="25"/>
+      <c r="E460" s="15"/>
       <c r="F460" s="15">
         <v>1</v>
       </c>
@@ -21213,6 +21671,7 @@
       </c>
       <c r="C461" s="25"/>
       <c r="D461" s="25"/>
+      <c r="E461" s="15"/>
       <c r="F461" s="15">
         <v>1</v>
       </c>
@@ -21255,6 +21714,7 @@
       </c>
       <c r="C462" s="25"/>
       <c r="D462" s="25"/>
+      <c r="E462" s="15"/>
       <c r="F462" s="15">
         <v>1</v>
       </c>
@@ -21297,6 +21757,7 @@
       </c>
       <c r="C463" s="25"/>
       <c r="D463" s="25"/>
+      <c r="E463" s="15"/>
       <c r="F463" s="15">
         <v>1</v>
       </c>
@@ -21339,6 +21800,7 @@
       </c>
       <c r="C464" s="25"/>
       <c r="D464" s="25"/>
+      <c r="E464" s="15"/>
       <c r="F464" s="15">
         <v>1</v>
       </c>
@@ -21381,6 +21843,7 @@
       </c>
       <c r="C465" s="25"/>
       <c r="D465" s="25"/>
+      <c r="E465" s="15"/>
       <c r="F465" s="15">
         <v>1</v>
       </c>
@@ -21423,6 +21886,7 @@
       </c>
       <c r="C466" s="25"/>
       <c r="D466" s="25"/>
+      <c r="E466" s="15"/>
       <c r="F466" s="15">
         <v>1</v>
       </c>
@@ -21465,6 +21929,7 @@
       </c>
       <c r="C467" s="25"/>
       <c r="D467" s="25"/>
+      <c r="E467" s="15"/>
       <c r="F467" s="15">
         <v>1</v>
       </c>
@@ -21507,6 +21972,7 @@
       </c>
       <c r="C468" s="25"/>
       <c r="D468" s="25"/>
+      <c r="E468" s="15"/>
       <c r="F468" s="15">
         <v>1</v>
       </c>
@@ -21549,6 +22015,7 @@
       </c>
       <c r="C469" s="25"/>
       <c r="D469" s="25"/>
+      <c r="E469" s="15"/>
       <c r="F469" s="15">
         <v>1</v>
       </c>
@@ -21591,6 +22058,7 @@
       </c>
       <c r="C470" s="25"/>
       <c r="D470" s="25"/>
+      <c r="E470" s="15"/>
       <c r="F470" s="15">
         <v>1</v>
       </c>
@@ -21633,6 +22101,7 @@
       </c>
       <c r="C471" s="25"/>
       <c r="D471" s="25"/>
+      <c r="E471" s="15"/>
       <c r="F471" s="15">
         <v>1</v>
       </c>
@@ -21675,6 +22144,7 @@
       </c>
       <c r="C472" s="25"/>
       <c r="D472" s="25"/>
+      <c r="E472" s="15"/>
       <c r="F472" s="15">
         <v>1</v>
       </c>
@@ -21717,6 +22187,7 @@
       </c>
       <c r="C473" s="25"/>
       <c r="D473" s="25"/>
+      <c r="E473" s="15"/>
       <c r="F473" s="15">
         <v>1</v>
       </c>
@@ -21759,6 +22230,7 @@
       </c>
       <c r="C474" s="25"/>
       <c r="D474" s="25"/>
+      <c r="E474" s="15"/>
       <c r="F474" s="15">
         <v>1</v>
       </c>
@@ -21801,6 +22273,7 @@
       </c>
       <c r="C475" s="25"/>
       <c r="D475" s="25"/>
+      <c r="E475" s="15"/>
       <c r="F475" s="15">
         <v>1</v>
       </c>
@@ -21843,6 +22316,7 @@
       </c>
       <c r="C476" s="25"/>
       <c r="D476" s="25"/>
+      <c r="E476" s="15"/>
       <c r="F476" s="15">
         <v>1</v>
       </c>
@@ -21885,6 +22359,7 @@
       </c>
       <c r="C477" s="25"/>
       <c r="D477" s="25"/>
+      <c r="E477" s="15"/>
       <c r="F477" s="15">
         <v>1</v>
       </c>
@@ -21927,6 +22402,7 @@
       </c>
       <c r="C478" s="25"/>
       <c r="D478" s="25"/>
+      <c r="E478" s="15"/>
       <c r="F478" s="15">
         <v>1</v>
       </c>
@@ -21969,6 +22445,7 @@
       </c>
       <c r="C479" s="25"/>
       <c r="D479" s="25"/>
+      <c r="E479" s="15"/>
       <c r="F479" s="15">
         <v>1</v>
       </c>
@@ -22011,6 +22488,7 @@
       </c>
       <c r="C480" s="25"/>
       <c r="D480" s="25"/>
+      <c r="E480" s="15"/>
       <c r="F480" s="15">
         <v>1</v>
       </c>
@@ -22053,6 +22531,7 @@
       </c>
       <c r="C481" s="25"/>
       <c r="D481" s="25"/>
+      <c r="E481" s="15"/>
       <c r="F481" s="15">
         <v>1</v>
       </c>
@@ -22095,6 +22574,7 @@
       </c>
       <c r="C482" s="25"/>
       <c r="D482" s="25"/>
+      <c r="E482" s="15"/>
       <c r="F482" s="15">
         <v>1</v>
       </c>
@@ -22137,6 +22617,7 @@
       </c>
       <c r="C483" s="25"/>
       <c r="D483" s="25"/>
+      <c r="E483" s="15"/>
       <c r="F483" s="15">
         <v>1</v>
       </c>
@@ -22179,6 +22660,7 @@
       </c>
       <c r="C484" s="25"/>
       <c r="D484" s="25"/>
+      <c r="E484" s="15"/>
       <c r="F484" s="15">
         <v>1</v>
       </c>
@@ -22221,6 +22703,7 @@
       </c>
       <c r="C485" s="25"/>
       <c r="D485" s="25"/>
+      <c r="E485" s="15"/>
       <c r="F485" s="15">
         <v>1</v>
       </c>
@@ -22263,6 +22746,7 @@
       </c>
       <c r="C486" s="25"/>
       <c r="D486" s="25"/>
+      <c r="E486" s="15"/>
       <c r="F486" s="15">
         <v>1</v>
       </c>
@@ -22305,6 +22789,7 @@
       </c>
       <c r="C487" s="25"/>
       <c r="D487" s="25"/>
+      <c r="E487" s="15"/>
       <c r="F487" s="15">
         <v>1</v>
       </c>
@@ -22347,6 +22832,7 @@
       </c>
       <c r="C488" s="25"/>
       <c r="D488" s="25"/>
+      <c r="E488" s="15"/>
       <c r="F488" s="15">
         <v>1</v>
       </c>
@@ -22389,6 +22875,7 @@
       </c>
       <c r="C489" s="25"/>
       <c r="D489" s="25"/>
+      <c r="E489" s="15"/>
       <c r="F489" s="15">
         <v>1</v>
       </c>
@@ -22431,6 +22918,7 @@
       </c>
       <c r="C490" s="25"/>
       <c r="D490" s="25"/>
+      <c r="E490" s="15"/>
       <c r="F490" s="15">
         <v>1</v>
       </c>
@@ -22473,6 +22961,7 @@
       </c>
       <c r="C491" s="25"/>
       <c r="D491" s="25"/>
+      <c r="E491" s="15"/>
       <c r="F491" s="15">
         <v>1</v>
       </c>
@@ -22515,6 +23004,7 @@
       </c>
       <c r="C492" s="25"/>
       <c r="D492" s="25"/>
+      <c r="E492" s="15"/>
       <c r="F492" s="15">
         <v>1</v>
       </c>
@@ -22557,6 +23047,7 @@
       </c>
       <c r="C493" s="25"/>
       <c r="D493" s="25"/>
+      <c r="E493" s="15"/>
       <c r="F493" s="15">
         <v>1</v>
       </c>
@@ -22599,6 +23090,7 @@
       </c>
       <c r="C494" s="25"/>
       <c r="D494" s="25"/>
+      <c r="E494" s="15"/>
       <c r="F494" s="15">
         <v>1</v>
       </c>
@@ -22641,6 +23133,7 @@
       </c>
       <c r="C495" s="25"/>
       <c r="D495" s="25"/>
+      <c r="E495" s="15"/>
       <c r="F495" s="15">
         <v>1</v>
       </c>
@@ -22683,6 +23176,7 @@
       </c>
       <c r="C496" s="25"/>
       <c r="D496" s="25"/>
+      <c r="E496" s="15"/>
       <c r="F496" s="15">
         <v>1</v>
       </c>
@@ -22725,6 +23219,7 @@
       </c>
       <c r="C497" s="25"/>
       <c r="D497" s="25"/>
+      <c r="E497" s="15"/>
       <c r="F497" s="15">
         <v>1</v>
       </c>
@@ -22767,6 +23262,7 @@
       </c>
       <c r="C498" s="25"/>
       <c r="D498" s="25"/>
+      <c r="E498" s="15"/>
       <c r="F498" s="15">
         <v>1</v>
       </c>
@@ -22809,6 +23305,7 @@
       </c>
       <c r="C499" s="25"/>
       <c r="D499" s="25"/>
+      <c r="E499" s="15"/>
       <c r="F499" s="15">
         <v>1</v>
       </c>
@@ -22851,6 +23348,7 @@
       </c>
       <c r="C500" s="25"/>
       <c r="D500" s="25"/>
+      <c r="E500" s="15"/>
       <c r="F500" s="15">
         <v>1</v>
       </c>
@@ -22893,6 +23391,7 @@
       </c>
       <c r="C501" s="25"/>
       <c r="D501" s="25"/>
+      <c r="E501" s="15"/>
       <c r="F501" s="15">
         <v>1</v>
       </c>
@@ -22935,6 +23434,7 @@
       </c>
       <c r="C502" s="25"/>
       <c r="D502" s="25"/>
+      <c r="E502" s="15"/>
       <c r="F502" s="15">
         <v>1</v>
       </c>
@@ -22977,7 +23477,7 @@
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="Q1:R1"/>
   </mergeCells>
-  <dataValidations count="520">
+  <dataValidations count="522">
     <dataValidation type="textLength" operator="greaterThan" showErrorMessage="1" errorStyle="stop" errorTitle="Required" error="PO_Number cannot be blank" sqref="A10:A502">
       <formula1>0</formula1>
     </dataValidation>
@@ -22995,6 +23495,12 @@
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" showInputMessage="1" promptTitle="Date format" prompt="DD/MM/YYYY" showErrorMessage="1" errorStyle="stop" errorTitle="Invalid date" error="Enter a valid date (DD/MM/YYYY)" sqref="C3:D502">
       <formula1>43831</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThan" showErrorMessage="1" errorStyle="stop" errorTitle="Booking Units required" error="Enter a whole number greater than 0 (no decimals)" sqref="E10:E502">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThan" showErrorMessage="1" errorStyle="stop" errorTitle="Booking Units required" error="Enter a whole number greater than 0 (no decimals)" sqref="E3:E502">
+      <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="greaterThan" showErrorMessage="1" errorStyle="stop" errorTitle="No of Cartons required" error="Enter a whole number greater than 0" sqref="F10:F502">
       <formula1>0</formula1>

</xml_diff>